<commit_message>
Update I3C test plan artifacts
</commit_message>
<xml_diff>
--- a/docs/test_plan/I3C_Testplan.xlsx
+++ b/docs/test_plan/I3C_Testplan.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="817">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -59,7 +59,7 @@
 Stimulus / Actions: Read `HC_CONTROL`, `HC_STATUS`, all timing registers, `QUEUE_STATUS`, and DAT[0..15].</t>
   </si>
   <si>
-    <t xml:space="preserve">Enable is 0; FSM idle/status reflects idle; queue flags show empty; DAT entries are 0; timing defaults match RTL.</t>
+    <t xml:space="preserve">Enable is 0; FSM idle/status reflects idle; queue flags show empty; DAT entries are 0; timing defaults match the CSR/module specification.</t>
   </si>
   <si>
     <t xml:space="preserve">High</t>
@@ -380,7 +380,7 @@
 Stimulus / Actions: Instantiate `sync_fifo` with non-power-of-two depth in a negative compile test.</t>
   </si>
   <si>
-    <t xml:space="preserve">Elaboration fatal/assertion occurs as implemented.</t>
+    <t xml:space="preserve">Elaboration fails with the documented parameter-check fatal/assertion required by the FIFO contract.</t>
   </si>
   <si>
     <t xml:space="preserve">Low</t>
@@ -600,7 +600,7 @@
 Stimulus / Actions: Observe `sel_od_pp_o` through address, ACK, data, T-bit, START/STOP.</t>
   </si>
   <si>
-    <t xml:space="preserve">OD is used for START/address/ACK/STOP and ENTDAA; PP is used only for implemented I3C SDR data phases.</t>
+    <t xml:space="preserve">OD is used for START/address/ACK/STOP and ENTDAA; PP is used only for in-scope MIPI I3C SDR data phases.</t>
   </si>
   <si>
     <t xml:space="preserve">`controller_active`, `flow_active`, `i3c_phy`</t>
@@ -612,23 +612,23 @@
     <t xml:space="preserve">BUS_011</t>
   </si>
   <si>
-    <t xml:space="preserve">Document current pad model limitation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`tb_pad_model_limit_check`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: Top-level UVM TB.
-Stimulus / Actions: Observe bus while `sel_od_pp_o` is active.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test records that `tb_i3c_top` models DUT pins as open-drain and leaves `sel_od_pp_o` unconnected; true pad-level PP verification needs TB enhancement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`tb_i3c_top`, `i3c_phy`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_tb_limitation`</t>
+    <t xml:space="preserve">Verify enhanced TB pad-model wiring for SDA drive/release and OD/PP visibility.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`tb_pad_model_odpp_wiring`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: Top-level UVM TB with `sda_oe_o` and `sel_od_pp_o` connected.
+Stimulus / Actions: Observe `sda_oe_o`, `sda_o`, `sel_od_pp_o`, and `sda_bus` during existing I3C write/read traffic; later extend with a dedicated OD/PP pad vseq.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`tb_i3c_top` drives SDA only when `sda_oe_o=1`, releases SDA when `sda_oe_o=0`, and exposes DUT pad signals through `i3c_if`; existing smoke/write/read regressions show no SDA contention. Dedicated phase-level PP checks remain future work.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`tb_i3c_top`, `i3c_if`, `i3c_phy`, `i3c_controller_top`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_pad_model`, `cp_sda_oe`, `cp_tb_odpp_visibility`</t>
   </si>
   <si>
     <t xml:space="preserve">I3C SDR Private Write</t>
@@ -637,7 +637,7 @@
     <t xml:space="preserve">SDRW_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Preserve existing write regression.</t>
+    <t xml:space="preserve">Verify baseline 4-byte SDR private write.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_regular_write_4b_existing`</t>
@@ -647,7 +647,7 @@
 Stimulus / Actions: Run `i3c_write_vseq` with TX word `DEAD_BEEF`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bus write uses dynamic address+W; data byte order is little-endian from TX word; RESP success length 4.</t>
+    <t xml:space="preserve">Bus write uses dynamic address+W; data byte order follows the project TX FIFO packing contract; RESP success length 4.</t>
   </si>
   <si>
     <t xml:space="preserve">Full DUT, UVM scoreboard</t>
@@ -713,7 +713,7 @@
 Stimulus / Actions: Send data bytes with even and odd parity.</t>
   </si>
   <si>
-    <t xml:space="preserve">T-bit equals odd parity generation used by RTL (`~^data_byte`) for every write byte.</t>
+    <t xml:space="preserve">T-bit makes the 8-bit data byte plus T-bit odd parity, equivalent to `~^data_byte`, for every write byte.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `bus_tx_flow`</t>
@@ -769,20 +769,20 @@
     <t xml:space="preserve">SDRW_007</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify no STOP when `toc=0`.</t>
+    <t xml:space="preserve">Verify SDR regular write continuation when `toc=0`.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_write_toc_zero`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Device ACKs; next command is queued as applicable.
-Stimulus / Actions: Issue write with `toc=0`.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RESP is produced without STOP only if current RTL/spec defines continuation; otherwise behavior is recorded as a spec gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_toc`</t>
+    <t xml:space="preserve">Preconditions: I3C device ACKs; a second SDR regular I3C command is already queued.
+Stimulus / Actions: Queue first write with `toc=0` and second write with `toc=1`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First write completes data/T-bit then emits `Sr` instead of STOP; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; both RESPs report success with matching TID/length.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_toc`, `cp_rstart_continuation`</t>
   </si>
   <si>
     <t xml:space="preserve">SDRW_008</t>
@@ -813,7 +813,7 @@
     <t xml:space="preserve">SDRR_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Preserve existing read regression.</t>
+    <t xml:space="preserve">Verify baseline 4-byte SDR private read.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_regular_read_4b_existing`</t>
@@ -823,7 +823,7 @@
 Stimulus / Actions: Run `i3c_read_vseq`.</t>
   </si>
   <si>
-    <t xml:space="preserve">RX FIFO word is `32'hBEBA_FECA`; RESP success length 4.</t>
+    <t xml:space="preserve">RX FIFO word matches the target bytes packed by the project RX FIFO contract, e.g. `32'hBEBA_FECA` for the existing stimulus; RESP success length 4.</t>
   </si>
   <si>
     <t xml:space="preserve">SDRR_002</t>
@@ -956,7 +956,7 @@
 Stimulus / Actions: Run read where final T-bit is 0.</t>
   </si>
   <si>
-    <t xml:space="preserve">Controller treats T-bit=0 as end/short-read indicator, not as parity error. `Parity` response is not expected in current RTL.</t>
+    <t xml:space="preserve">Per I3C SDR read semantics, T-bit=0 is an end-of-data indicator, not a parity error; response is Success if the requested length is met, otherwise `I3cShortReadErr`.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`</t>
@@ -965,13 +965,35 @@
     <t xml:space="preserve">`cp_read_tbit`, `cp_resp_err`</t>
   </si>
   <si>
+    <t xml:space="preserve">SDRR_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify SDR regular read continuation when `toc=0`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i3c_read_toc_zero`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: I3C device returns requested read data; a second SDR regular I3C command is already queued.
+Stimulus / Actions: Queue first read with `toc=0` and second write with `toc=1`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First read completes requested data/T-bit then emits `Sr` instead of STOP; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; RX data and both RESPs match expected length/TID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active`, `scl_generator`, `bus_rx_flow`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_toc`, `cp_rstart_continuation`, `cp_dir_read_to_write`</t>
+  </si>
+  <si>
     <t xml:space="preserve">Immediate Data Transfer</t>
   </si>
   <si>
     <t xml:space="preserve">IMM_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Preserve existing immediate smoke.</t>
+    <t xml:space="preserve">Verify baseline immediate write descriptor flow.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_immediate_write_smoke_existing`</t>
@@ -981,7 +1003,7 @@
 Stimulus / Actions: Run `i3c_smoke_vseq`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Two inline data bytes are transmitted; RESP success.</t>
+    <t xml:space="preserve">Two inline data bytes are transmitted according to descriptor `dtt` and project packing rules; RESP success.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `bus_tx_flow`, UVM</t>
@@ -1015,20 +1037,20 @@
     <t xml:space="preserve">IMM_003</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify immediate STOP control.</t>
+    <t xml:space="preserve">Verify immediate `toc` policy.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_immediate_write_toc`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Target ACKs.
+    <t xml:space="preserve">Preconditions: Target ACKs; immediate `toc=0` continuation policy is not specified for the current project descriptor set.
 Stimulus / Actions: Repeat immediate command with `toc=1` and `toc=0`.</t>
   </si>
   <si>
-    <t xml:space="preserve">`toc=1` generates STOP; `toc=0` behavior matches RTL/spec or is documented as a gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_toc`, `cp_imm`</t>
+    <t xml:space="preserve">`toc=1` generates STOP and success. `toc=0` is a clarification/negative case until the project spec defines immediate continuation; acceptable sign-off behavior must be one specified policy such as reject/abort with error or forced STOP, and the bus must not hang without STOP or `Sr`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_toc`, `cp_imm`, `cp_unsupported_policy`</t>
   </si>
   <si>
     <t xml:space="preserve">IMM_004</t>
@@ -1059,11 +1081,11 @@
     <t xml:space="preserve">`immediate_addr_nack`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Target NACKs address.
+    <t xml:space="preserve">Preconditions: Target NACKs the address ACK/NACK slot.
 Stimulus / Actions: Issue I3C and I2C immediate writes.</t>
   </si>
   <si>
-    <t xml:space="preserve">No data phase after NACK; RESP error is `AddrHeader`; controller returns idle.</t>
+    <t xml:space="preserve">Controller generates STOP immediately after address NACK; no inline data byte is transmitted; RESP error is `AddrHeader` with length 0.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_resp_err`, `cross_imm_x_device_type`</t>
@@ -1082,7 +1104,7 @@
 Stimulus / Actions: Issue multi-byte I2C immediate write.</t>
   </si>
   <si>
-    <t xml:space="preserve">RESP error is `Nack`; transfer stops/recover behavior follows RTL/spec.</t>
+    <t xml:space="preserve">Controller generates STOP after data NACK; no later inline data byte is transmitted; RESP error is `Nack`.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_data_ack`, `cp_resp_err`</t>
@@ -1100,11 +1122,11 @@
     <t xml:space="preserve">`ccc_entdaa_opening_frame`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: AddressAssignment CMD queued; device ACKs broadcast header and CCC.
+    <t xml:space="preserve">Preconditions: AddressAssignment CMD queued; targets ACK the broadcast header.
 Stimulus / Actions: Issue `AddressAssignment` with `cmd=0x07`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bus shows START, `7'h7E+W`, ACK, `8'h07`, ACK before ENTDAA rounds.</t>
+    <t xml:space="preserve">Bus shows START, `7'h7E+W`, broadcast-header ACK, ENTDAA opcode `8'h07` with T-bit odd parity, then the ENTDAA `7'h7E+R` round sequence.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `bus_tx_flow`, `bus_rx_flow`</t>
@@ -1116,41 +1138,44 @@
     <t xml:space="preserve">CCC_002</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify broadcast ENEC frame generation as implemented.</t>
+    <t xml:space="preserve">Verify broadcast ENEC frame generation.</t>
   </si>
   <si>
     <t xml:space="preserve">`ccc_broadcast_enec_frame`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Immediate CMD with `cp=1`, `cmd=8'h00`; target ACKs.
-Stimulus / Actions: Send event byte/defining data according to descriptor convention.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bus frame matches current ENEC implementation; any missing defining-byte behavior is recorded as implementation gap.</t>
+    <t xml:space="preserve">Preconditions: Immediate CMD with `cp=1`, `cmd=8'h00`; target ACKs only the broadcast header.
+Stimulus / Actions: Send Target Events byte in `def_or_data_byte1` according to the immediate descriptor convention.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus shows START, `7'h7E+W` in open-drain, broadcast-header ACK in open-drain, ENEC opcode `8'h00` in push-pull, opcode T-bit `~^8'h00`, Target Events byte in push-pull, event-byte T-bit `~^event_byte`, and STOP. No target ACK is expected after the CCC opcode or event byte.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `i3c_monitor`</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_ccc_opcode`, `cp_ccc_broadcast`, `cp_odpp_phase`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCC_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify broadcast DISEC frame generation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`ccc_broadcast_disec_frame`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: Immediate CMD with `cp=1`, `cmd=8'h01`; target ACKs the broadcast header.
+Stimulus / Actions: Send Target Events byte according to the project descriptor convention.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus frame follows the MIPI broadcast DISEC format: START, `7'h7E+W`, broadcast-header ACK, DISEC opcode `8'h01` with T-bit, Target Events byte with T-bit, then STOP; ENTDAA controller is not activated.</t>
+  </si>
+  <si>
     <t xml:space="preserve">`cp_ccc_opcode`, `cp_ccc_broadcast`</t>
   </si>
   <si>
-    <t xml:space="preserve">CCC_003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify broadcast DISEC frame generation as implemented.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`ccc_broadcast_disec_frame`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: Immediate CMD with `cp=1`, `cmd=8'h01`; target ACKs.
-Stimulus / Actions: Send event byte/defining data according to descriptor convention.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bus frame matches current DISEC implementation; no ENTDAA controller activation.</t>
-  </si>
-  <si>
     <t xml:space="preserve">CCC_004</t>
   </si>
   <si>
@@ -1160,11 +1185,11 @@
     <t xml:space="preserve">`ccc_direct_enec_frame`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: DAT dynamic address valid; target ACKs broadcast and direct address.
+    <t xml:space="preserve">Preconditions: DAT dynamic address valid; target ACKs broadcast header and direct address.
 Stimulus / Actions: Immediate CMD with `cp=1`, `cmd=8'h80`, one data byte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bus shows broadcast header, CCC, Sr, target dynamic address+W, data/T-bit, STOP.</t>
+    <t xml:space="preserve">Bus shows broadcast header, CCC opcode/T-bit, Sr, target dynamic address+W, address ACK, data/T-bit, STOP.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_ccc_direct`, `cp_rstart`</t>
@@ -1179,11 +1204,11 @@
     <t xml:space="preserve">`ccc_direct_disec_frame`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: DAT dynamic address valid; target ACKs.
+    <t xml:space="preserve">Preconditions: DAT dynamic address valid; target ACKs broadcast header and direct address.
 Stimulus / Actions: Immediate CMD with `cp=1`, `cmd=8'h81`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Direct DISEC frame is emitted; RESP success if all ACKs are received.</t>
+    <t xml:space="preserve">Direct DISEC frame is emitted with CCC opcode/T-bit, Sr, direct address ACK, optional data/T-bit as specified; RESP success if all required address ACKs are received.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_ccc_opcode`, `cp_ccc_direct`</t>
@@ -1198,11 +1223,11 @@
     <t xml:space="preserve">`ccc_broadcast_header_nack`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Device NACKs `7'h7E+W` or CCC byte ACK slot.
+    <t xml:space="preserve">Preconditions: Device NACKs `7'h7E+W`.
 Stimulus / Actions: Issue ENEC/DISEC/ENTDAA command.</t>
   </si>
   <si>
-    <t xml:space="preserve">Controller reports an implemented error status or the gap is documented; no hang is allowed for sign-off.</t>
+    <t xml:space="preserve">Controller reports the specified address/header error, generates legal bus recovery, and does not send CCC payload after broadcast-header NACK.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, RESP FIFO</t>
@@ -1220,11 +1245,11 @@
     <t xml:space="preserve">`ccc_direct_target_nack`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Target ACKs broadcast header and CCC, NACKs direct address.
+    <t xml:space="preserve">Preconditions: Target ACKs broadcast header, observes the direct CCC opcode/T-bit, and NACKs direct address.
 Stimulus / Actions: Issue direct ENEC/DISEC.</t>
   </si>
   <si>
-    <t xml:space="preserve">No direct data byte is sent after address NACK; RESP and bus recovery match RTL/spec.</t>
+    <t xml:space="preserve">No direct data byte is sent after address NACK; RESP and bus recovery match the address/header NACK policy in the project spec.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_ccc_direct`, `cp_addr_ack`</t>
@@ -1243,7 +1268,7 @@
 Stimulus / Actions: Issue representative unsupported broadcast and direct opcodes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current RTL lacks explicit opcode validation; expected result is documented behavior or a required `NotSupported` enhancement.</t>
+    <t xml:space="preserve">This is a clarification/negative test until the project spec defines unsupported CCC handling. Required sign-off behavior should be a specified `NotSupported`/error response or software restriction; the controller must not emit an undefined successful CCC frame, corrupt queues, or lock up.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `i3c_pkg`</t>
@@ -1268,7 +1293,7 @@
 Stimulus / Actions: Issue AddressAssignment with `dev_idx=0`, `dev_count=1`.</t>
   </si>
   <si>
-    <t xml:space="preserve">ENTDAA frame completes; assigned address byte uses correct parity; RESP success; RX visibility follows implemented policy.</t>
+    <t xml:space="preserve">ENTDAA frame completes per MIPI sequence; assigned address byte uses correct parity; target ACKs the assignment; RESP success; any software-visible DAA result follows the documented project format.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `entdaa_controller`, `entdaa_fsm`</t>
@@ -1397,7 +1422,7 @@
 Stimulus / Actions: Run successful ENTDAA.</t>
   </si>
   <si>
-    <t xml:space="preserve">Internal captured PID/BCR/DCR match target; software-visible RX data format is verified against RTL or documented as spec gap.</t>
+    <t xml:space="preserve">Captured PID/BCR/DCR match the bits driven by the target in the MIPI ENTDAA order; software-visible RX data is checked only after its project format is specified.</t>
   </si>
   <si>
     <t xml:space="preserve">`entdaa_fsm`, `flow_active`, RX FIFO</t>
@@ -1419,7 +1444,7 @@
 Stimulus / Actions: Run `dev_idx=15`, `dev_count=1`, then `dev_idx=15`, `dev_count&gt;1`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Single entry works; out-of-range case follows current saturation behavior or is documented as SW responsibility.</t>
+    <t xml:space="preserve">Single entry works; out-of-range `dev_idx+dev_count` is a clarification/negative case that must either produce a specified error or be forbidden by a documented software precondition.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_dat_boundary`</t>
@@ -1438,7 +1463,7 @@
 Stimulus / Actions: Interrupt during PID/BCR/DCR reception.</t>
   </si>
   <si>
-    <t xml:space="preserve">ENTDAA terminates to Done/NoDev path and controller returns idle or gap is documented.</t>
+    <t xml:space="preserve">ENTDAA exits through a specified abort/recovery policy and controller returns to a legal idle/recoverable state; if no policy exists, this is a spec gap and not positive sign-off coverage.</t>
   </si>
   <si>
     <t xml:space="preserve">`entdaa_fsm`, `entdaa_controller`, `bus_monitor`</t>
@@ -1567,7 +1592,7 @@
 Stimulus / Actions: Issue multi-byte write.</t>
   </si>
   <si>
-    <t xml:space="preserve">Transfer stops or recovers according to RTL/spec; RESP error is `Nack`; next legal transfer passes.</t>
+    <t xml:space="preserve">Transfer stops after the NACKed byte per I2C/project error policy; RESP error is `Nack`; next legal transfer passes.</t>
   </si>
   <si>
     <t xml:space="preserve">I2C_006</t>
@@ -1649,7 +1674,7 @@
 Stimulus / Actions: Run I3C write/read, I2C write/read, and direct CCC address phases.</t>
   </si>
   <si>
-    <t xml:space="preserve">RESP error is `AddrHeader` where current RTL supports it; no data phase after address NACK.</t>
+    <t xml:space="preserve">RESP error is `AddrHeader` for every supported command class with an address/header NACK; no data phase occurs after address NACK.</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_003</t>
@@ -1697,7 +1722,7 @@
 Stimulus / Actions: Attempt CRC, Frame, Ovl, HcAborted, NotSupported, Parity scenarios.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current RTL has no production paths for these codes; results are N/A or enhancement requests, not expected positive coverage.</t>
+    <t xml:space="preserve">Error codes outside the specified controller scope are N/A or enhancement requests, not positive coverage; any in-scope error code must have a spec-derived stimulus and expected response.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_pkg`, `flow_active`</t>
@@ -1779,7 +1804,7 @@
 Stimulus / Actions: Assert `HC_CONTROL[1]` while not idle.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current spec says this is undefined; test documents behavior and recommends SW only reset when `FSM_IDLE=1`.</t>
+    <t xml:space="preserve">If the spec leaves this undefined, the test records a spec gap and recommends SW only reset when `FSM_IDLE=1`; it is not positive sign-off coverage until a busy-reset policy is specified.</t>
   </si>
   <si>
     <t xml:space="preserve">`csr_registers`, `hci_queues`, `flow_active`</t>
@@ -1801,7 +1826,7 @@
 Stimulus / Actions: Hold SCL low during transfer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current design has no complete bus recovery/timeout; test should fail by timeout or document gap.</t>
+    <t xml:space="preserve">If no timeout/recovery requirement is specified in the project scope, this is a documented N/A/gap; it must not be treated as a functional pass merely because the controller waits forever.</t>
   </si>
   <si>
     <t xml:space="preserve">`scl_generator`, `bus_monitor`</t>
@@ -1889,7 +1914,7 @@
 Stimulus / Actions: Inject STOP-like SDA rise while SCL high during DAA or data phase.</t>
   </si>
   <si>
-    <t xml:space="preserve">Implemented modules terminate or test records missing recovery behavior.</t>
+    <t xml:space="preserve">Controller follows a specified abort/recovery policy; if none exists, the test records a spec gap and is not positive sign-off coverage.</t>
   </si>
   <si>
     <t xml:space="preserve">`bus_monitor`, `flow_active`, `entdaa_controller`</t>
@@ -1911,7 +1936,7 @@
 Stimulus / Actions: Queue command while SCL/SDA not both high.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current RTL behavior is documented; if unsupported, SW precondition must require idle bus before command.</t>
+    <t xml:space="preserve">Controller must either wait for the specified Bus Available/Idle condition or reject the command with a specified error/software precondition; observed RTL behavior alone is not a pass criterion.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_bus_busy_start`</t>
@@ -2364,6 +2389,9 @@
   </si>
   <si>
     <t xml:space="preserve">zero, all-one, alternating A/5, walking-one, random</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_toc`</t>
   </si>
   <si>
     <t xml:space="preserve">0, 1</t>
@@ -3485,7 +3513,7 @@
         <v>194</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>118</v>
+        <v>52</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>195</v>
@@ -4008,39 +4036,39 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B45" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="B45" t="s" s="2">
+      <c r="C45" t="s" s="2">
         <v>304</v>
       </c>
-      <c r="C45" t="s" s="2">
+      <c r="D45" t="s" s="2">
         <v>305</v>
       </c>
-      <c r="D45" t="s" s="2">
+      <c r="E45" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="F45" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="E45" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="F45" t="s" s="2">
+      <c r="G45" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="G45" t="s" s="2">
+      <c r="H45" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="I45" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="H45" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I45" t="s" s="2">
+      <c r="J45" t="s" s="2">
         <v>309</v>
-      </c>
-      <c r="J45" t="s" s="2">
-        <v>310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>19</v>
+        <v>310</v>
       </c>
       <c r="B46" t="s" s="2">
         <v>311</v>
@@ -4093,13 +4121,13 @@
         <v>322</v>
       </c>
       <c r="H47" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I47" t="s" s="2">
-        <v>160</v>
+        <v>323</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="48">
@@ -4107,31 +4135,31 @@
         <v>19</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C48" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D48" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="E48" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="E48" t="s" s="2">
-        <v>325</v>
-      </c>
       <c r="F48" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H48" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I48" t="s" s="2">
-        <v>224</v>
+        <v>160</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="49">
@@ -4139,31 +4167,31 @@
         <v>19</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D49" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="E49" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="E49" t="s" s="2">
-        <v>331</v>
-      </c>
       <c r="F49" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I49" t="s" s="2">
-        <v>283</v>
+        <v>224</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="50">
@@ -4171,36 +4199,36 @@
         <v>19</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D50" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="E50" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="E50" t="s" s="2">
-        <v>337</v>
-      </c>
       <c r="F50" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I50" t="s" s="2">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="J50" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>342</v>
+        <v>19</v>
       </c>
       <c r="B51" t="s" s="2">
         <v>343</v>
@@ -4224,15 +4252,15 @@
         <v>16</v>
       </c>
       <c r="I51" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="J51" t="s" s="2">
         <v>348</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>349</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>19</v>
+        <v>349</v>
       </c>
       <c r="B52" t="s" s="2">
         <v>350</v>
@@ -4288,10 +4316,10 @@
         <v>16</v>
       </c>
       <c r="I53" t="s" s="2">
-        <v>301</v>
+        <v>362</v>
       </c>
       <c r="J53" t="s" s="2">
-        <v>356</v>
+        <v>363</v>
       </c>
     </row>
     <row r="54">
@@ -4299,31 +4327,31 @@
         <v>19</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C54" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D54" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E54" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="F54" t="s" s="2">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I54" t="s" s="2">
-        <v>160</v>
+        <v>301</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="55">
@@ -4331,31 +4359,31 @@
         <v>19</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C55" t="s" s="2">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D55" t="s" s="2">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E55" t="s" s="2">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F55" t="s" s="2">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I55" t="s" s="2">
-        <v>301</v>
+        <v>160</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="56">
@@ -4363,31 +4391,31 @@
         <v>19</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C56" t="s" s="2">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D56" t="s" s="2">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E56" t="s" s="2">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F56" t="s" s="2">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I56" t="s" s="2">
-        <v>379</v>
+        <v>301</v>
       </c>
       <c r="J56" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="57">
@@ -4395,31 +4423,31 @@
         <v>19</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C57" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D57" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="E57" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="E57" t="s" s="2">
-        <v>382</v>
-      </c>
       <c r="F57" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I57" t="s" s="2">
-        <v>301</v>
+        <v>387</v>
       </c>
       <c r="J57" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="58">
@@ -4427,36 +4455,36 @@
         <v>19</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D58" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="E58" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F58" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="H58" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I58" t="s" s="2">
-        <v>392</v>
+        <v>301</v>
       </c>
       <c r="J58" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>394</v>
+        <v>19</v>
       </c>
       <c r="B59" t="s" s="2">
         <v>395</v>
@@ -4477,7 +4505,7 @@
         <v>399</v>
       </c>
       <c r="H59" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I59" t="s" s="2">
         <v>400</v>
@@ -4488,34 +4516,34 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>19</v>
+        <v>402</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C60" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D60" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="E60" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="E60" t="s" s="2">
-        <v>403</v>
-      </c>
       <c r="F60" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J60" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="61">
@@ -4523,31 +4551,31 @@
         <v>19</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C61" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D61" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="E61" t="s" s="2">
         <v>411</v>
       </c>
-      <c r="E61" t="s" s="2">
-        <v>410</v>
-      </c>
       <c r="F61" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G61" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H61" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I61" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J61" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="62">
@@ -4555,31 +4583,31 @@
         <v>19</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C62" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D62" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="E62" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="E62" t="s" s="2">
-        <v>417</v>
-      </c>
       <c r="F62" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I62" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J62" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="63">
@@ -4587,31 +4615,31 @@
         <v>19</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C63" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D63" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="E63" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="E63" t="s" s="2">
-        <v>424</v>
-      </c>
       <c r="F63" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G63" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="H63" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I63" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J63" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="64">
@@ -4619,31 +4647,31 @@
         <v>19</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C64" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D64" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="E64" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="E64" t="s" s="2">
-        <v>431</v>
-      </c>
       <c r="F64" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I64" t="s" s="2">
-        <v>407</v>
+        <v>436</v>
       </c>
       <c r="J64" t="s" s="2">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="65">
@@ -4651,31 +4679,31 @@
         <v>19</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C65" t="s" s="2">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D65" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E65" t="s" s="2">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="F65" t="s" s="2">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G65" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H65" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I65" t="s" s="2">
-        <v>441</v>
+        <v>415</v>
       </c>
       <c r="J65" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="66">
@@ -4683,31 +4711,31 @@
         <v>19</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C66" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D66" t="s" s="2">
+        <v>446</v>
+      </c>
+      <c r="E66" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="E66" t="s" s="2">
-        <v>444</v>
-      </c>
       <c r="F66" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="H66" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I66" t="s" s="2">
-        <v>421</v>
+        <v>449</v>
       </c>
       <c r="J66" t="s" s="2">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="67">
@@ -4715,31 +4743,31 @@
         <v>19</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C67" t="s" s="2">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D67" t="s" s="2">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E67" t="s" s="2">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F67" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G67" t="s" s="2">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="H67" t="s" s="2">
         <v>52</v>
       </c>
       <c r="I67" t="s" s="2">
-        <v>454</v>
+        <v>429</v>
       </c>
       <c r="J67" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="68">
@@ -4747,25 +4775,25 @@
         <v>19</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C68" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D68" t="s" s="2">
+        <v>459</v>
+      </c>
+      <c r="E68" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="E68" t="s" s="2">
-        <v>457</v>
-      </c>
       <c r="F68" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="H68" t="s" s="2">
-        <v>461</v>
+        <v>52</v>
       </c>
       <c r="I68" t="s" s="2">
         <v>462</v>
@@ -4776,28 +4804,28 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B69" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="B69" t="s" s="2">
+      <c r="C69" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="C69" t="s" s="2">
+      <c r="D69" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="D69" t="s" s="2">
+      <c r="E69" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="F69" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="E69" t="s" s="2">
-        <v>466</v>
-      </c>
-      <c r="F69" t="s" s="2">
+      <c r="G69" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="G69" t="s" s="2">
+      <c r="H69" t="s" s="2">
         <v>469</v>
-      </c>
-      <c r="H69" t="s" s="2">
-        <v>16</v>
       </c>
       <c r="I69" t="s" s="2">
         <v>470</v>
@@ -4808,34 +4836,34 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>19</v>
+        <v>472</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C70" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D70" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="E70" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="E70" t="s" s="2">
-        <v>473</v>
-      </c>
       <c r="F70" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G70" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="H70" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I70" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J70" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="71">
@@ -4843,31 +4871,31 @@
         <v>19</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C71" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D71" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="E71" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="E71" t="s" s="2">
-        <v>480</v>
-      </c>
       <c r="F71" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G71" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="H71" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I71" t="s" s="2">
-        <v>264</v>
+        <v>485</v>
       </c>
       <c r="J71" t="s" s="2">
-        <v>265</v>
+        <v>486</v>
       </c>
     </row>
     <row r="72">
@@ -4875,31 +4903,31 @@
         <v>19</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="C72" t="s" s="2">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D72" t="s" s="2">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="E72" t="s" s="2">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F72" t="s" s="2">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G72" t="s" s="2">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="H72" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I72" t="s" s="2">
-        <v>283</v>
+        <v>264</v>
       </c>
       <c r="J72" t="s" s="2">
-        <v>489</v>
+        <v>265</v>
       </c>
     </row>
     <row r="73">
@@ -4907,31 +4935,31 @@
         <v>19</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C73" t="s" s="2">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D73" t="s" s="2">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E73" t="s" s="2">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F73" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I73" t="s" s="2">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="J73" t="s" s="2">
-        <v>341</v>
+        <v>497</v>
       </c>
     </row>
     <row r="74">
@@ -4939,31 +4967,31 @@
         <v>19</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="C74" t="s" s="2">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="D74" t="s" s="2">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="E74" t="s" s="2">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="F74" t="s" s="2">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I74" t="s" s="2">
-        <v>500</v>
+        <v>301</v>
       </c>
       <c r="J74" t="s" s="2">
-        <v>501</v>
+        <v>348</v>
       </c>
     </row>
     <row r="75">
@@ -4971,36 +4999,36 @@
         <v>19</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C75" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D75" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="E75" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="E75" t="s" s="2">
-        <v>503</v>
-      </c>
       <c r="F75" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="G75" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="H75" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I75" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="J75" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>509</v>
+        <v>19</v>
       </c>
       <c r="B76" t="s" s="2">
         <v>510</v>
@@ -5021,45 +5049,45 @@
         <v>514</v>
       </c>
       <c r="H76" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I76" t="s" s="2">
-        <v>379</v>
+        <v>515</v>
       </c>
       <c r="J76" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>19</v>
+        <v>517</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C77" t="s" s="2">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D77" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E77" t="s" s="2">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F77" t="s" s="2">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G77" t="s" s="2">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="H77" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I77" t="s" s="2">
-        <v>301</v>
+        <v>387</v>
       </c>
       <c r="J77" t="s" s="2">
-        <v>232</v>
+        <v>523</v>
       </c>
     </row>
     <row r="78">
@@ -5067,22 +5095,22 @@
         <v>19</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="C78" t="s" s="2">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D78" t="s" s="2">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E78" t="s" s="2">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="F78" t="s" s="2">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="G78" t="s" s="2">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="H78" t="s" s="2">
         <v>16</v>
@@ -5091,7 +5119,7 @@
         <v>301</v>
       </c>
       <c r="J78" t="s" s="2">
-        <v>341</v>
+        <v>232</v>
       </c>
     </row>
     <row r="79">
@@ -5099,22 +5127,22 @@
         <v>19</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="C79" t="s" s="2">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="D79" t="s" s="2">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="E79" t="s" s="2">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="F79" t="s" s="2">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="G79" t="s" s="2">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="H79" t="s" s="2">
         <v>16</v>
@@ -5123,7 +5151,7 @@
         <v>301</v>
       </c>
       <c r="J79" t="s" s="2">
-        <v>271</v>
+        <v>348</v>
       </c>
     </row>
     <row r="80">
@@ -5131,31 +5159,31 @@
         <v>19</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="C80" t="s" s="2">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="D80" t="s" s="2">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="E80" t="s" s="2">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="F80" t="s" s="2">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="G80" t="s" s="2">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="H80" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I80" t="s" s="2">
-        <v>536</v>
+        <v>301</v>
       </c>
       <c r="J80" t="s" s="2">
-        <v>537</v>
+        <v>271</v>
       </c>
     </row>
     <row r="81">
@@ -5163,31 +5191,31 @@
         <v>19</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C81" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D81" t="s" s="2">
+        <v>541</v>
+      </c>
+      <c r="E81" t="s" s="2">
         <v>540</v>
       </c>
-      <c r="E81" t="s" s="2">
-        <v>539</v>
-      </c>
       <c r="F81" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="G81" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="H81" t="s" s="2">
-        <v>16</v>
+        <v>118</v>
       </c>
       <c r="I81" t="s" s="2">
-        <v>264</v>
+        <v>544</v>
       </c>
       <c r="J81" t="s" s="2">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="82">
@@ -5195,31 +5223,31 @@
         <v>19</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C82" t="s" s="2">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D82" t="s" s="2">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E82" t="s" s="2">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F82" t="s" s="2">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="G82" t="s" s="2">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="H82" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I82" t="s" s="2">
-        <v>549</v>
+        <v>264</v>
       </c>
       <c r="J82" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="83">
@@ -5227,31 +5255,31 @@
         <v>19</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C83" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D83" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="E83" t="s" s="2">
         <v>553</v>
       </c>
-      <c r="E83" t="s" s="2">
-        <v>552</v>
-      </c>
       <c r="F83" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G83" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="H83" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I83" t="s" s="2">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="J83" t="s" s="2">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="84">
@@ -5259,31 +5287,31 @@
         <v>19</v>
       </c>
       <c r="B84" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="C84" t="s" s="2">
+        <v>560</v>
+      </c>
+      <c r="D84" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="E84" t="s" s="2">
+        <v>560</v>
+      </c>
+      <c r="F84" t="s" s="2">
+        <v>562</v>
+      </c>
+      <c r="G84" t="s" s="2">
+        <v>563</v>
+      </c>
+      <c r="H84" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I84" t="s" s="2">
         <v>557</v>
       </c>
-      <c r="C84" t="s" s="2">
-        <v>558</v>
-      </c>
-      <c r="D84" t="s" s="2">
-        <v>559</v>
-      </c>
-      <c r="E84" t="s" s="2">
-        <v>558</v>
-      </c>
-      <c r="F84" t="s" s="2">
-        <v>560</v>
-      </c>
-      <c r="G84" t="s" s="2">
-        <v>561</v>
-      </c>
-      <c r="H84" t="s" s="2">
-        <v>52</v>
-      </c>
-      <c r="I84" t="s" s="2">
-        <v>562</v>
-      </c>
       <c r="J84" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="85">
@@ -5291,31 +5319,31 @@
         <v>19</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C85" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D85" t="s" s="2">
+        <v>567</v>
+      </c>
+      <c r="E85" t="s" s="2">
         <v>566</v>
       </c>
-      <c r="E85" t="s" s="2">
-        <v>565</v>
-      </c>
       <c r="F85" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G85" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="H85" t="s" s="2">
         <v>52</v>
       </c>
       <c r="I85" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="J85" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="86">
@@ -5323,36 +5351,36 @@
         <v>19</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C86" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="D86" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="E86" t="s" s="2">
         <v>573</v>
       </c>
-      <c r="E86" t="s" s="2">
-        <v>572</v>
-      </c>
       <c r="F86" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="G86" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="H86" t="s" s="2">
         <v>52</v>
       </c>
       <c r="I86" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="J86" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>578</v>
+        <v>19</v>
       </c>
       <c r="B87" t="s" s="2">
         <v>579</v>
@@ -5373,7 +5401,7 @@
         <v>583</v>
       </c>
       <c r="H87" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I87" t="s" s="2">
         <v>584</v>
@@ -5384,34 +5412,34 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>19</v>
+        <v>586</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C88" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D88" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="E88" t="s" s="2">
         <v>588</v>
       </c>
-      <c r="E88" t="s" s="2">
-        <v>587</v>
-      </c>
       <c r="F88" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="G88" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="H88" t="s" s="2">
-        <v>461</v>
+        <v>16</v>
       </c>
       <c r="I88" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="J88" t="s" s="2">
-        <v>463</v>
+        <v>593</v>
       </c>
     </row>
     <row r="89">
@@ -5419,31 +5447,31 @@
         <v>19</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="C89" t="s" s="2">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D89" t="s" s="2">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E89" t="s" s="2">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="F89" t="s" s="2">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="G89" t="s" s="2">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="H89" t="s" s="2">
-        <v>52</v>
+        <v>469</v>
       </c>
       <c r="I89" t="s" s="2">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="J89" t="s" s="2">
-        <v>598</v>
+        <v>471</v>
       </c>
     </row>
     <row r="90">
@@ -5451,60 +5479,60 @@
         <v>19</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C90" t="s" s="2">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D90" t="s" s="2">
+        <v>602</v>
+      </c>
+      <c r="E90" t="s" s="2">
         <v>601</v>
       </c>
-      <c r="E90" t="s" s="2">
-        <v>600</v>
-      </c>
       <c r="F90" t="s" s="2">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="G90" t="s" s="2">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H90" t="s" s="2">
         <v>52</v>
       </c>
       <c r="I90" t="s" s="2">
-        <v>569</v>
+        <v>605</v>
       </c>
       <c r="J90" t="s" s="2">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>605</v>
+        <v>19</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C91" t="s" s="2">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="D91" t="s" s="2">
+        <v>609</v>
+      </c>
+      <c r="E91" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="E91" t="s" s="2">
-        <v>607</v>
-      </c>
       <c r="F91" t="s" s="2">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G91" t="s" s="2">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="H91" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I91" t="s" s="2">
-        <v>611</v>
+        <v>577</v>
       </c>
       <c r="J91" t="s" s="2">
         <v>612</v>
@@ -5512,34 +5540,34 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>19</v>
+        <v>613</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C92" t="s" s="2">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D92" t="s" s="2">
+        <v>616</v>
+      </c>
+      <c r="E92" t="s" s="2">
         <v>615</v>
       </c>
-      <c r="E92" t="s" s="2">
-        <v>614</v>
-      </c>
       <c r="F92" t="s" s="2">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="G92" t="s" s="2">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="H92" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I92" t="s" s="2">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="J92" t="s" s="2">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="93">
@@ -5547,31 +5575,31 @@
         <v>19</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C93" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D93" t="s" s="2">
+        <v>623</v>
+      </c>
+      <c r="E93" t="s" s="2">
         <v>622</v>
       </c>
-      <c r="E93" t="s" s="2">
-        <v>621</v>
-      </c>
       <c r="F93" t="s" s="2">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="G93" t="s" s="2">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H93" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I93" t="s" s="2">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="J93" t="s" s="2">
-        <v>619</v>
+        <v>627</v>
       </c>
     </row>
     <row r="94">
@@ -5579,31 +5607,31 @@
         <v>19</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C94" t="s" s="2">
+        <v>629</v>
+      </c>
+      <c r="D94" t="s" s="2">
+        <v>630</v>
+      </c>
+      <c r="E94" t="s" s="2">
+        <v>629</v>
+      </c>
+      <c r="F94" t="s" s="2">
+        <v>631</v>
+      </c>
+      <c r="G94" t="s" s="2">
+        <v>632</v>
+      </c>
+      <c r="H94" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I94" t="s" s="2">
+        <v>633</v>
+      </c>
+      <c r="J94" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="D94" t="s" s="2">
-        <v>628</v>
-      </c>
-      <c r="E94" t="s" s="2">
-        <v>627</v>
-      </c>
-      <c r="F94" t="s" s="2">
-        <v>629</v>
-      </c>
-      <c r="G94" t="s" s="2">
-        <v>630</v>
-      </c>
-      <c r="H94" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I94" t="s" s="2">
-        <v>631</v>
-      </c>
-      <c r="J94" t="s" s="2">
-        <v>632</v>
       </c>
     </row>
     <row r="95">
@@ -5611,31 +5639,31 @@
         <v>19</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C95" t="s" s="2">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D95" t="s" s="2">
+        <v>636</v>
+      </c>
+      <c r="E95" t="s" s="2">
         <v>635</v>
       </c>
-      <c r="E95" t="s" s="2">
-        <v>634</v>
-      </c>
       <c r="F95" t="s" s="2">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="H95" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I95" t="s" s="2">
-        <v>631</v>
+        <v>639</v>
       </c>
       <c r="J95" t="s" s="2">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="96">
@@ -5643,31 +5671,31 @@
         <v>19</v>
       </c>
       <c r="B96" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="C96" t="s" s="2">
+        <v>642</v>
+      </c>
+      <c r="D96" t="s" s="2">
+        <v>643</v>
+      </c>
+      <c r="E96" t="s" s="2">
+        <v>642</v>
+      </c>
+      <c r="F96" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="G96" t="s" s="2">
+        <v>645</v>
+      </c>
+      <c r="H96" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="I96" t="s" s="2">
         <v>639</v>
       </c>
-      <c r="C96" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="D96" t="s" s="2">
-        <v>641</v>
-      </c>
-      <c r="E96" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="F96" t="s" s="2">
-        <v>642</v>
-      </c>
-      <c r="G96" t="s" s="2">
-        <v>643</v>
-      </c>
-      <c r="H96" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I96" t="s" s="2">
-        <v>644</v>
-      </c>
       <c r="J96" t="s" s="2">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="97">
@@ -5675,31 +5703,31 @@
         <v>19</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C97" t="s" s="2">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D97" t="s" s="2">
+        <v>649</v>
+      </c>
+      <c r="E97" t="s" s="2">
         <v>648</v>
       </c>
-      <c r="E97" t="s" s="2">
-        <v>647</v>
-      </c>
       <c r="F97" t="s" s="2">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G97" t="s" s="2">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="H97" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I97" t="s" s="2">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="J97" t="s" s="2">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="98">
@@ -5707,36 +5735,36 @@
         <v>19</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C98" t="s" s="2">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D98" t="s" s="2">
+        <v>656</v>
+      </c>
+      <c r="E98" t="s" s="2">
         <v>655</v>
       </c>
-      <c r="E98" t="s" s="2">
-        <v>654</v>
-      </c>
       <c r="F98" t="s" s="2">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G98" t="s" s="2">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="H98" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I98" t="s" s="2">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="J98" t="s" s="2">
-        <v>659</v>
+        <v>660</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>660</v>
+        <v>19</v>
       </c>
       <c r="B99" t="s" s="2">
         <v>661</v>
@@ -5757,7 +5785,7 @@
         <v>665</v>
       </c>
       <c r="H99" t="s" s="2">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="I99" t="s" s="2">
         <v>666</v>
@@ -5768,34 +5796,34 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>19</v>
+        <v>668</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C100" t="s" s="2">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D100" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="E100" t="s" s="2">
         <v>670</v>
       </c>
-      <c r="E100" t="s" s="2">
-        <v>669</v>
-      </c>
       <c r="F100" t="s" s="2">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G100" t="s" s="2">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="H100" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I100" t="s" s="2">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="J100" t="s" s="2">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="101">
@@ -5803,31 +5831,31 @@
         <v>19</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C101" t="s" s="2">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D101" t="s" s="2">
+        <v>678</v>
+      </c>
+      <c r="E101" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="E101" t="s" s="2">
-        <v>676</v>
-      </c>
       <c r="F101" t="s" s="2">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="G101" t="s" s="2">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="H101" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I101" t="s" s="2">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="102">
@@ -5835,31 +5863,31 @@
         <v>19</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="C102" t="s" s="2">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="D102" t="s" s="2">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="E102" t="s" s="2">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="F102" t="s" s="2">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="G102" t="s" s="2">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="H102" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I102" t="s" s="2">
-        <v>686</v>
+        <v>674</v>
       </c>
       <c r="J102" t="s" s="2">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="103">
@@ -5867,31 +5895,31 @@
         <v>19</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C103" t="s" s="2">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D103" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="E103" t="s" s="2">
         <v>690</v>
       </c>
-      <c r="E103" t="s" s="2">
-        <v>689</v>
-      </c>
       <c r="F103" t="s" s="2">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G103" t="s" s="2">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="H103" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I103" t="s" s="2">
-        <v>666</v>
+        <v>694</v>
       </c>
       <c r="J103" t="s" s="2">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="104">
@@ -5899,31 +5927,31 @@
         <v>19</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="C104" t="s" s="2">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D104" t="s" s="2">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E104" t="s" s="2">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="F104" t="s" s="2">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="G104" t="s" s="2">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="H104" t="s" s="2">
-        <v>118</v>
+        <v>52</v>
       </c>
       <c r="I104" t="s" s="2">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="105">
@@ -5931,31 +5959,31 @@
         <v>19</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="C105" t="s" s="2">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="D105" t="s" s="2">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="E105" t="s" s="2">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="F105" t="s" s="2">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="G105" t="s" s="2">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="H105" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I105" t="s" s="2">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="J105" t="s" s="2">
-        <v>699</v>
+        <v>707</v>
       </c>
     </row>
     <row r="106">
@@ -5963,60 +5991,60 @@
         <v>19</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="C106" t="s" s="2">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="D106" t="s" s="2">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="E106" t="s" s="2">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="F106" t="s" s="2">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="G106" t="s" s="2">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="H106" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I106" t="s" s="2">
-        <v>160</v>
+        <v>674</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>710</v>
+        <v>707</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>711</v>
+        <v>19</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C107" t="s" s="2">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="D107" t="s" s="2">
+        <v>715</v>
+      </c>
+      <c r="E107" t="s" s="2">
         <v>714</v>
       </c>
-      <c r="E107" t="s" s="2">
-        <v>713</v>
-      </c>
       <c r="F107" t="s" s="2">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="G107" t="s" s="2">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="H107" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I107" t="s" s="2">
-        <v>717</v>
+        <v>160</v>
       </c>
       <c r="J107" t="s" s="2">
         <v>718</v>
@@ -6024,34 +6052,34 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>19</v>
+        <v>719</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C108" t="s" s="2">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D108" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="E108" t="s" s="2">
         <v>721</v>
       </c>
-      <c r="E108" t="s" s="2">
-        <v>720</v>
-      </c>
       <c r="F108" t="s" s="2">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="H108" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I108" t="s" s="2">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="J108" t="s" s="2">
-        <v>718</v>
+        <v>726</v>
       </c>
     </row>
     <row r="109">
@@ -6059,31 +6087,31 @@
         <v>19</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="C109" t="s" s="2">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="D109" t="s" s="2">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="E109" t="s" s="2">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="F109" t="s" s="2">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="H109" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I109" t="s" s="2">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="J109" t="s" s="2">
-        <v>718</v>
+        <v>726</v>
       </c>
     </row>
     <row r="110">
@@ -6091,31 +6119,63 @@
         <v>19</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C110" t="s" s="2">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D110" t="s" s="2">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="E110" t="s" s="2">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="F110" t="s" s="2">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="G110" t="s" s="2">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="H110" t="s" s="2">
         <v>118</v>
       </c>
       <c r="I110" t="s" s="2">
-        <v>536</v>
+        <v>737</v>
       </c>
       <c r="J110" t="s" s="2">
-        <v>718</v>
+        <v>726</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B111" t="s" s="2">
+        <v>738</v>
+      </c>
+      <c r="C111" t="s" s="2">
+        <v>739</v>
+      </c>
+      <c r="D111" t="s" s="2">
+        <v>740</v>
+      </c>
+      <c r="E111" t="s" s="2">
+        <v>739</v>
+      </c>
+      <c r="F111" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="G111" t="s" s="2">
+        <v>742</v>
+      </c>
+      <c r="H111" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="I111" t="s" s="2">
+        <v>544</v>
+      </c>
+      <c r="J111" t="s" s="2">
+        <v>726</v>
       </c>
     </row>
   </sheetData>
@@ -6127,18 +6187,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>736</v>
+        <v>744</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>737</v>
+        <v>745</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>19</v>
@@ -6152,10 +6212,10 @@
         <v>19</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>740</v>
+        <v>748</v>
       </c>
     </row>
     <row r="4">
@@ -6163,10 +6223,10 @@
         <v>19</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>742</v>
+        <v>750</v>
       </c>
     </row>
     <row r="5">
@@ -6174,10 +6234,10 @@
         <v>19</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>744</v>
+        <v>752</v>
       </c>
     </row>
     <row r="6">
@@ -6185,10 +6245,10 @@
         <v>19</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>746</v>
+        <v>754</v>
       </c>
     </row>
     <row r="7">
@@ -6199,7 +6259,7 @@
         <v>218</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>747</v>
+        <v>755</v>
       </c>
     </row>
     <row r="8">
@@ -6207,10 +6267,10 @@
         <v>19</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>245</v>
+        <v>756</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>748</v>
+        <v>757</v>
       </c>
     </row>
     <row r="9">
@@ -6218,10 +6278,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>749</v>
+        <v>758</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>750</v>
+        <v>759</v>
       </c>
     </row>
     <row r="10">
@@ -6229,10 +6289,10 @@
         <v>19</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>751</v>
+        <v>760</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>752</v>
+        <v>761</v>
       </c>
     </row>
     <row r="11">
@@ -6240,10 +6300,10 @@
         <v>19</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>753</v>
+        <v>762</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>754</v>
+        <v>763</v>
       </c>
     </row>
     <row r="12">
@@ -6251,10 +6311,10 @@
         <v>19</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>755</v>
+        <v>764</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>756</v>
+        <v>765</v>
       </c>
     </row>
     <row r="13">
@@ -6265,7 +6325,7 @@
         <v>225</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>757</v>
+        <v>766</v>
       </c>
     </row>
     <row r="14">
@@ -6273,10 +6333,10 @@
         <v>19</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>758</v>
+        <v>767</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>759</v>
+        <v>768</v>
       </c>
     </row>
     <row r="15">
@@ -6284,10 +6344,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>760</v>
+        <v>769</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>761</v>
+        <v>770</v>
       </c>
     </row>
     <row r="16">
@@ -6295,10 +6355,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>762</v>
+        <v>771</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>763</v>
+        <v>772</v>
       </c>
     </row>
     <row r="17">
@@ -6306,10 +6366,10 @@
         <v>19</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>764</v>
+        <v>773</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>765</v>
+        <v>774</v>
       </c>
     </row>
     <row r="18">
@@ -6320,7 +6380,7 @@
         <v>134</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>766</v>
+        <v>775</v>
       </c>
     </row>
     <row r="19">
@@ -6331,7 +6391,7 @@
         <v>189</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>767</v>
+        <v>776</v>
       </c>
     </row>
     <row r="20">
@@ -6339,10 +6399,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>768</v>
+        <v>777</v>
       </c>
     </row>
     <row r="21">
@@ -6353,7 +6413,7 @@
         <v>161</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>769</v>
+        <v>778</v>
       </c>
     </row>
     <row r="22">
@@ -6361,10 +6421,10 @@
         <v>19</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>770</v>
+        <v>779</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>771</v>
+        <v>780</v>
       </c>
     </row>
     <row r="23">
@@ -6372,10 +6432,10 @@
         <v>19</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>772</v>
+        <v>781</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>773</v>
+        <v>782</v>
       </c>
     </row>
     <row r="24">
@@ -6383,10 +6443,10 @@
         <v>19</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>774</v>
+        <v>783</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>775</v>
+        <v>784</v>
       </c>
     </row>
     <row r="25">
@@ -6394,10 +6454,10 @@
         <v>19</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>776</v>
+        <v>785</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>777</v>
+        <v>786</v>
       </c>
     </row>
     <row r="26">
@@ -6405,10 +6465,10 @@
         <v>19</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>778</v>
+        <v>787</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>779</v>
+        <v>788</v>
       </c>
     </row>
     <row r="27">
@@ -6416,10 +6476,10 @@
         <v>19</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>780</v>
+        <v>789</v>
       </c>
     </row>
     <row r="28">
@@ -6435,7 +6495,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>781</v>
+        <v>790</v>
       </c>
       <c r="B29" t="s" s="2">
         <v>19</v>
@@ -6449,10 +6509,10 @@
         <v>19</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>782</v>
+        <v>791</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>783</v>
+        <v>792</v>
       </c>
     </row>
     <row r="31">
@@ -6460,10 +6520,10 @@
         <v>19</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>784</v>
+        <v>793</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>785</v>
+        <v>794</v>
       </c>
     </row>
     <row r="32">
@@ -6471,10 +6531,10 @@
         <v>19</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>786</v>
+        <v>795</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>787</v>
+        <v>796</v>
       </c>
     </row>
     <row r="33">
@@ -6482,10 +6542,10 @@
         <v>19</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>788</v>
+        <v>797</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>789</v>
+        <v>798</v>
       </c>
     </row>
     <row r="34">
@@ -6493,10 +6553,10 @@
         <v>19</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>790</v>
+        <v>799</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>791</v>
+        <v>800</v>
       </c>
     </row>
     <row r="35">
@@ -6504,10 +6564,10 @@
         <v>19</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>792</v>
+        <v>801</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>793</v>
+        <v>802</v>
       </c>
     </row>
     <row r="36">
@@ -6515,10 +6575,10 @@
         <v>19</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>794</v>
+        <v>803</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>795</v>
+        <v>804</v>
       </c>
     </row>
     <row r="37">
@@ -6526,10 +6586,10 @@
         <v>19</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>796</v>
+        <v>805</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>797</v>
+        <v>806</v>
       </c>
     </row>
     <row r="38">
@@ -6537,10 +6597,10 @@
         <v>19</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>798</v>
+        <v>807</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>799</v>
+        <v>808</v>
       </c>
     </row>
     <row r="39">
@@ -6548,10 +6608,10 @@
         <v>19</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>800</v>
+        <v>809</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>801</v>
+        <v>810</v>
       </c>
     </row>
   </sheetData>
@@ -6566,43 +6626,43 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>802</v>
+        <v>811</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>803</v>
+        <v>812</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>804</v>
+        <v>813</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>698</v>
+        <v>706</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>805</v>
+        <v>814</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>704</v>
+        <v>712</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>806</v>
+        <v>815</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>709</v>
+        <v>717</v>
       </c>
     </row>
   </sheetData>
@@ -6626,58 +6686,58 @@
         <v>4</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>807</v>
+        <v>816</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>699</v>
+        <v>707</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>699</v>
+        <v>707</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>710</v>
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SDR flow DV and SVA coverage
</commit_message>
<xml_diff>
--- a/docs/test_plan/I3C_Testplan.xlsx
+++ b/docs/test_plan/I3C_Testplan.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="854">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -99,6 +99,28 @@
     <t xml:space="preserve">CSR_003</t>
   </si>
   <si>
+    <t xml:space="preserve">Verify broadcast-header control bit read/write behavior and both private-transfer bus-framing modes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`csr_broadcast_header_control`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: Controller idle and CMD FIFO empty; DAT[0] is I3C dynamic address `0x08`; device ACKs target address and, when enabled, broadcast header.
+Stimulus / Actions: Read `HC_CONTROL[BROADCAST_ADDR_ENABLE]` after reset; set and clear the bit through `HC_CONTROL`; set only this bit without `HC_CONTROL[0]`; then issue one 4-byte SDR private write with `BROADCAST_ADDR_ENABLE=0` and one with `BROADCAST_ADDR_ENABLE=1`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reset value is 0; writable set/clear behavior is correct; setting `BROADCAST_ADDR_ENABLE` alone does not enable the controller and does not start a bus transaction; disabled write starts directly with `START + 0x08/W`; enabled write emits `START + 0x7e/W + ACK + Sr + 0x08/W + ACK + data/T-bit + STOP`; both RESPs report success with matching lengths.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`csr_registers`, `flow_active`, `scl_generator`, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`, `cp_enable`, `cp_private_start_prefix`, `cp_first_address`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSR_004</t>
+  </si>
+  <si>
     <t xml:space="preserve">Verify timing register read/write behavior.</t>
   </si>
   <si>
@@ -106,16 +128,16 @@
   </si>
   <si>
     <t xml:space="preserve">Preconditions: Controller idle.
-Stimulus / Actions: Write/read `T_R` through `T_HD_DAT` using default, minimum nonzero, and random legal values.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Readback matches written `[19:0]` values; reserved upper bits read 0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_timing_reg`, `cp_timing_value`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSR_004</t>
+Stimulus / Actions: Write/read all I3C timing CSRs `T_R` through `T_BUS_FREE` and all I2C timing CSRs `I2C_T_R` through `I2C_T_BUF` using default, zero, minimum nonzero, maximum 20-bit, random legal, and reserved-upper-bit values.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readback matches written `[19:0]` values; reserved upper bits read 0; writes to one timing CSR do not alter other timing CSRs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_timing_reg`, `cp_timing_value`, `cr_timing_reg_value`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSR_005</t>
   </si>
   <si>
     <t xml:space="preserve">Verify all DAT entries and field packing.</t>
@@ -137,7 +159,7 @@
     <t xml:space="preserve">`cp_dat_idx`, `cp_device_type`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_005</t>
+    <t xml:space="preserve">CSR_006</t>
   </si>
   <si>
     <t xml:space="preserve">Verify 64-bit CMD staging from two 32-bit writes.</t>
@@ -159,7 +181,7 @@
     <t xml:space="preserve">`cp_cmd_staging`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_006</t>
+    <t xml:space="preserve">CSR_007</t>
   </si>
   <si>
     <t xml:space="preserve">Verify partial CMD staging is not disturbed by unrelated CSR writes.</t>
@@ -184,7 +206,7 @@
     <t xml:space="preserve">`cp_cmd_staging`, `cp_csr_interleave`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_007</t>
+    <t xml:space="preserve">CSR_008</t>
   </si>
   <si>
     <t xml:space="preserve">Verify software reset flushes queues.</t>
@@ -203,7 +225,7 @@
     <t xml:space="preserve">`cp_sw_reset`, `cp_fifo_state`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_008</t>
+    <t xml:space="preserve">CSR_009</t>
   </si>
   <si>
     <t xml:space="preserve">Verify stale DWORD0 cannot corrupt a later command.</t>
@@ -222,7 +244,7 @@
     <t xml:space="preserve">`cp_sw_reset`, `cp_cmd_staging`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_009</t>
+    <t xml:space="preserve">CSR_010</t>
   </si>
   <si>
     <t xml:space="preserve">Verify full/empty status bits.</t>
@@ -244,7 +266,7 @@
     <t xml:space="preserve">`cp_fifo_kind`, `cp_fifo_state`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_010</t>
+    <t xml:space="preserve">CSR_011</t>
   </si>
   <si>
     <t xml:space="preserve">Verify RX/RESP port pop behavior.</t>
@@ -263,7 +285,7 @@
     <t xml:space="preserve">`cp_port_pop`, `cp_empty_read`</t>
   </si>
   <si>
-    <t xml:space="preserve">CSR_011</t>
+    <t xml:space="preserve">CSR_012</t>
   </si>
   <si>
     <t xml:space="preserve">Verify unmapped address behavior.</t>
@@ -502,23 +524,23 @@
     <t xml:space="preserve">BUS_006</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify clock stall behavior.</t>
+    <t xml:space="preserve">Verify clock stall behavior while waiting for commands or legal backpressure conditions.</t>
   </si>
   <si>
     <t xml:space="preserve">`scl_waitcmd_stall_resume`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: TX FIFO or RX FIFO backpressure condition available.
-Stimulus / Actions: Force `StallWrite` or `StallRead`; later remove the stall.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCL is held low during wait and resumes without extra START/STOP or data corruption.</t>
+    <t xml:space="preserve">Preconditions: Controller is idle or in a supported wait condition.
+Stimulus / Actions: Hold the relevant wait condition, then release it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCL behavior remains legal and traffic resumes or terminates without data corruption.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `scl_generator`</t>
   </si>
   <si>
-    <t xml:space="preserve">`cp_stall_type`</t>
+    <t xml:space="preserve">`cp_wait_state`</t>
   </si>
   <si>
     <t xml:space="preserve">BUS_007</t>
@@ -637,45 +659,45 @@
     <t xml:space="preserve">SDRW_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify baseline 4-byte SDR private write.</t>
+    <t xml:space="preserve">Verify baseline 4-byte SDR private write without broadcast-header preamble.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_regular_write_4b_existing`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; device ACKs.
+    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; `HC_CONTROL[BROADCAST_ADDR_ENABLE]=0`; device ACKs.
 Stimulus / Actions: Run `i3c_write_vseq` with TX word `DEAD_BEEF`.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bus write uses dynamic address+W; data byte order follows the project TX FIFO packing contract; RESP success length 4.</t>
+    <t xml:space="preserve">Bus write starts with `START + 0x08/W + ACK`; no `0x7e` preamble is emitted; data byte order follows the project TX FIFO packing contract; RESP success length 4.</t>
   </si>
   <si>
     <t xml:space="preserve">Full DUT, UVM scoreboard</t>
   </si>
   <si>
-    <t xml:space="preserve">`cp_cmd_attr`, `cp_dir`, `cp_len_4`</t>
+    <t xml:space="preserve">`cp_cmd_attr`, `cp_dir`, `cp_len_4`, `cp_private_start_prefix`</t>
   </si>
   <si>
     <t xml:space="preserve">SDRW_002</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify write lengths and TX packing.</t>
+    <t xml:space="preserve">Verify write lengths, TX packing, and broadcast-header private-write framing.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_regular_write_len_sweep`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Device ACKs address and write data.
-Stimulus / Actions: Write lengths 1,2,3,4,5,7,8,16 using patterned TX words.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exact byte count transmitted; correct byte order; RESP length equals bytes transferred.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `hci_queues`, `bus_tx_flow`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_data_len`, `cp_tx_word_boundary`</t>
+    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; device ACKs address and write data; run once with `HC_CONTROL[BROADCAST_ADDR_ENABLE]=0` and once with it set.
+Stimulus / Actions: Write lengths 1,2,3,4,5,7,8,16 using patterned TX words in both private-address modes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exact byte count transmitted; correct byte order; RESP length equals bytes transferred; disabled mode starts directly with `START + 0x08/W`; enabled mode emits `START + 0x7e/W + ACK + Sr + 0x08/W` before data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active`, `hci_queues`, `bus_tx_flow`, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_data_len`, `cp_tx_word_boundary`, `cp_private_start_prefix`</t>
   </si>
   <si>
     <t xml:space="preserve">SDRW_003</t>
@@ -747,42 +769,45 @@
     <t xml:space="preserve">SDRW_006</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify TX underflow stall/recovery.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`i3c_write_tx_fifo_empty_stall`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: Write length exceeds initially available TX data.
-Stimulus / Actions: Issue write, delay additional TX data, then provide it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controller stalls without corrupting bus data and resumes when TX data is available.</t>
+    <t xml:space="preserve">Verify TX underflow error handling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i3c_write_tx_fifo_underflow_ovl`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: Write length exceeds available TX FIFO data.
+Stimulus / Actions: Issue an 8-byte write with only one TX DWORD available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controller transfers the available 4 bytes, does not enter old `StallWrite`, generates STOP, and writes RESP `Ovl` with response length 4.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `hci_queues`, `scl_generator`</t>
   </si>
   <si>
-    <t xml:space="preserve">`cp_stall_type`, `cp_tx_empty`</t>
+    <t xml:space="preserve">`cp_resp_err_ovl`, `cp_tx_empty`</t>
   </si>
   <si>
     <t xml:space="preserve">SDRW_007</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify SDR regular write continuation when `toc=0`.</t>
+    <t xml:space="preserve">Verify SDR regular write continuation when `toc=0`, including broadcast-header-enabled private continuation framing.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_write_toc_zero`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: I3C device ACKs; a second SDR regular I3C command is already queued.
+    <t xml:space="preserve">Preconditions: I3C device ACKs; a second SDR regular I3C command is already queued; run once with `HC_CONTROL[BROADCAST_ADDR_ENABLE]=0` and once with it set.
 Stimulus / Actions: Queue first write with `toc=0` and second write with `toc=1`.</t>
   </si>
   <si>
-    <t xml:space="preserve">First write completes data/T-bit then emits `Sr` instead of STOP; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; both RESPs report success with matching TID/length.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_toc`, `cp_rstart_continuation`</t>
+    <t xml:space="preserve">First write completes data/T-bit then emits `Sr` instead of STOP; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; both RESPs report success with matching TID/length. With broadcast-header enabled, the first private transfer emits `START + 0x7e/W + ACK + Sr + dynamic address`, and the continuation does not emit a second `0x7e` preamble.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active`, `scl_generator`, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`, `cp_toc`, `cp_rstart_continuation`, `cp_private_start_prefix`</t>
   </si>
   <si>
     <t xml:space="preserve">SDRW_008</t>
@@ -813,20 +838,42 @@
     <t xml:space="preserve">SDRR_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify baseline 4-byte SDR private read.</t>
+    <t xml:space="preserve">Verify baseline 4-byte SDR private read without broadcast-header preamble.</t>
   </si>
   <si>
     <t xml:space="preserve">`i3c_regular_read_4b_existing`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; target returns four bytes.
+    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; `HC_CONTROL[BROADCAST_ADDR_ENABLE]=0`; target returns four bytes.
 Stimulus / Actions: Run `i3c_read_vseq`.</t>
   </si>
   <si>
-    <t xml:space="preserve">RX FIFO word matches the target bytes packed by the project RX FIFO contract, e.g. `32'hBEBA_FECA` for the existing stimulus; RESP success length 4.</t>
+    <t xml:space="preserve">Bus read starts with `START + 0x08/R + ACK`; no `0x7e` preamble is emitted; RX FIFO word matches the target bytes packed by the project RX FIFO contract, e.g. `32'hBEBA_FECA` for the existing stimulus; RESP success length 4.</t>
   </si>
   <si>
     <t xml:space="preserve">SDRR_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify SDR private read with broadcast-header preamble enabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i3c_read_broadcast_header_enabled`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; `HC_CONTROL[BROADCAST_ADDR_ENABLE]=1`; target ACKs broadcast header and returns read data.
+Stimulus / Actions: Issue a 4-byte regular read.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus frame is `START + 0x7e/W + ACK + Sr + 0x08/R + ACK + read data/T-bit + STOP`; monitor/scoreboard treat the preamble and target phase as one complete transaction; RX data and RESP length match expected bytes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active`, `scl_generator`, `bus_rx_flow`, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`, `cp_private_start_prefix`, `cp_first_address`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDRR_003</t>
   </si>
   <si>
     <t xml:space="preserve">Verify read lengths and RX packing.</t>
@@ -848,7 +895,7 @@
     <t xml:space="preserve">`cp_data_len`, `cp_rx_partial_dword`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_003</t>
+    <t xml:space="preserve">SDRR_004</t>
   </si>
   <si>
     <t xml:space="preserve">Verify target early end handling.</t>
@@ -867,7 +914,7 @@
     <t xml:space="preserve">`cp_short_read`, `cp_resp_err`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_004</t>
+    <t xml:space="preserve">SDRR_005</t>
   </si>
   <si>
     <t xml:space="preserve">Verify controller termination at requested length.</t>
@@ -886,7 +933,7 @@
     <t xml:space="preserve">`cp_read_end_policy`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_005</t>
+    <t xml:space="preserve">SDRR_006</t>
   </si>
   <si>
     <t xml:space="preserve">Verify address NACK response on read.</t>
@@ -905,7 +952,7 @@
     <t xml:space="preserve">`flow_active`, `bus_rx_flow`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_006</t>
+    <t xml:space="preserve">SDRR_007</t>
   </si>
   <si>
     <t xml:space="preserve">Verify RX backpressure.</t>
@@ -924,7 +971,7 @@
     <t xml:space="preserve">`cp_rx_full`, `cp_stall_type`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_007</t>
+    <t xml:space="preserve">SDRR_008</t>
   </si>
   <si>
     <t xml:space="preserve">Verify read data integrity.</t>
@@ -943,7 +990,7 @@
     <t xml:space="preserve">`i3c_driver`, `bus_rx_flow`, scoreboard</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_008</t>
+    <t xml:space="preserve">SDRR_009</t>
   </si>
   <si>
     <t xml:space="preserve">Verify read T-bit semantics.</t>
@@ -965,7 +1012,7 @@
     <t xml:space="preserve">`cp_read_tbit`, `cp_resp_err`</t>
   </si>
   <si>
-    <t xml:space="preserve">SDRR_009</t>
+    <t xml:space="preserve">SDRR_010</t>
   </si>
   <si>
     <t xml:space="preserve">Verify SDR regular read continuation when `toc=0`.</t>
@@ -987,6 +1034,25 @@
     <t xml:space="preserve">`cp_toc`, `cp_rstart_continuation`, `cp_dir_read_to_write`</t>
   </si>
   <si>
+    <t xml:space="preserve">SDRR_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify broadcast-header preamble is not repeated across a private read continuation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i3c_read_toc_zero_broadcast_header_once`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: `HC_CONTROL[BROADCAST_ADDR_ENABLE]=1`; I3C device returns requested read data; a second SDR regular I3C command is already queued.
+Stimulus / Actions: Queue first read with `toc=0` and second command with `toc=1`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First command emits `START + 0x7e/W + ACK + Sr + dynamic address`; continuation after the repeated START does not emit a second `0x7e` preamble before the final STOP; RX data and RESPs remain correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`, `cp_toc`, `cp_private_start_prefix`</t>
+  </si>
+  <si>
     <t xml:space="preserve">Immediate Data Transfer</t>
   </si>
   <si>
@@ -1547,6 +1613,28 @@
     <t xml:space="preserve">I2C_003</t>
   </si>
   <si>
+    <t xml:space="preserve">Verify legacy I2C transfers ignore private-transfer broadcast-header control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i2c_broadcast_addr_enable_ignored`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: `HC_CONTROL[BROADCAST_ADDR_ENABLE]=1`; DAT[0].`device=1` with static address programmed; target ACKs.
+Stimulus / Actions: Run representative I2C read and write commands.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First address remains the DAT static address for both directions; no `0x7e` preamble is emitted; OD-only behavior and I2C ACK/NACK sequencing are unchanged.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active`, `scl_generator`, `bus_tx_flow`, `bus_rx_flow`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`, `cp_first_address`, `cp_i2c_dir`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2C_004</t>
+  </si>
+  <si>
     <t xml:space="preserve">Verify I2C read/write length behavior.</t>
   </si>
   <si>
@@ -1560,7 +1648,7 @@
     <t xml:space="preserve">Correct TX/RX packing; partial RX DWORD preserved; RESP length correct.</t>
   </si>
   <si>
-    <t xml:space="preserve">I2C_004</t>
+    <t xml:space="preserve">I2C_005</t>
   </si>
   <si>
     <t xml:space="preserve">Verify I2C address NACK.</t>
@@ -1579,7 +1667,7 @@
     <t xml:space="preserve">`cp_resp_err`, `cp_i2c_addr_ack`</t>
   </si>
   <si>
-    <t xml:space="preserve">I2C_005</t>
+    <t xml:space="preserve">I2C_006</t>
   </si>
   <si>
     <t xml:space="preserve">Verify I2C data-byte NACK.</t>
@@ -1595,7 +1683,7 @@
     <t xml:space="preserve">Transfer stops after the NACKed byte per I2C/project error policy; RESP error is `Nack`; next legal transfer passes.</t>
   </si>
   <si>
-    <t xml:space="preserve">I2C_006</t>
+    <t xml:space="preserve">I2C_007</t>
   </si>
   <si>
     <t xml:space="preserve">Verify legacy transfers remain open-drain.</t>
@@ -1617,7 +1705,7 @@
     <t xml:space="preserve">`cp_odpp_phase`, `cp_i2c`</t>
   </si>
   <si>
-    <t xml:space="preserve">I2C_007</t>
+    <t xml:space="preserve">I2C_008</t>
   </si>
   <si>
     <t xml:space="preserve">Verify configured I2C timing path.</t>
@@ -2382,6 +2470,24 @@
     <t xml:space="preserve">Write, Read</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_broadcast_addr_enable`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">disabled, enabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_private_start_prefix`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dynamic-address-first, broadcast-header-then-dynamic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_first_address`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`0x7e`, dynamic address, static address</t>
+  </si>
+  <si>
     <t xml:space="preserve">`cp_data_len`</t>
   </si>
   <si>
@@ -2457,6 +2563,9 @@
     <t xml:space="preserve">I3C SDR timing, I2C legacy timing, custom timing</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_stall_type`</t>
+  </si>
+  <si>
     <t xml:space="preserve">TX empty, RX full, RESP full, none</t>
   </si>
   <si>
@@ -2548,6 +2657,12 @@
   </si>
   <si>
     <t xml:space="preserve">Verify timing for START/STOP/Sr under I3C and I2C settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`broadcast_addr_enable x transaction_type x first_address`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ensure the control bit changes only private I3C first-address behavior while I2C, CCC, and ENTDAA retain their protocol-required address flows.</t>
   </si>
   <si>
     <t xml:space="preserve">`prev_cmd_attr x next_cmd_attr`</t>
@@ -2748,10 +2863,10 @@
         <v>16</v>
       </c>
       <c r="I4" t="s" s="2">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -2759,28 +2874,28 @@
         <v>19</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="E5" t="s" s="2">
-        <v>34</v>
-      </c>
       <c r="F5" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J5" t="s" s="2">
         <v>39</v>
@@ -2841,13 +2956,13 @@
         <v>51</v>
       </c>
       <c r="H7" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="I7" t="s" s="2">
+      <c r="J7" t="s" s="2">
         <v>53</v>
-      </c>
-      <c r="J7" t="s" s="2">
-        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -2855,31 +2970,31 @@
         <v>19</v>
       </c>
       <c r="B8" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="C8" t="s" s="2">
+      <c r="D8" t="s" s="2">
         <v>56</v>
       </c>
-      <c r="D8" t="s" s="2">
+      <c r="E8" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="E8" t="s" s="2">
-        <v>56</v>
-      </c>
-      <c r="F8" t="s" s="2">
+      <c r="G8" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="G8" t="s" s="2">
+      <c r="H8" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="H8" t="s" s="2">
-        <v>16</v>
-      </c>
       <c r="I8" t="s" s="2">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9">
@@ -2887,31 +3002,31 @@
         <v>19</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="E9" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="E9" t="s" s="2">
-        <v>62</v>
-      </c>
       <c r="F9" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I9" t="s" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10">
@@ -2919,28 +3034,28 @@
         <v>19</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="E10" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="E10" t="s" s="2">
-        <v>68</v>
-      </c>
       <c r="F10" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I10" t="s" s="2">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="J10" t="s" s="2">
         <v>73</v>
@@ -2972,10 +3087,10 @@
         <v>16</v>
       </c>
       <c r="I11" t="s" s="2">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="J11" t="s" s="2">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
@@ -2983,36 +3098,36 @@
         <v>19</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D12" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="E12" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="E12" t="s" s="2">
-        <v>81</v>
-      </c>
       <c r="F12" t="s" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H12" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="I12" t="s" s="2">
-        <v>17</v>
-      </c>
       <c r="J12" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s" s="2">
         <v>87</v>
@@ -3033,18 +3148,18 @@
         <v>91</v>
       </c>
       <c r="H13" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I13" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="J13" t="s" s="2">
         <v>92</v>
-      </c>
-      <c r="J13" t="s" s="2">
-        <v>93</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>94</v>
@@ -3097,13 +3212,13 @@
         <v>105</v>
       </c>
       <c r="H15" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I15" t="s" s="2">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16">
@@ -3111,31 +3226,31 @@
         <v>19</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D16" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="E16" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="E16" t="s" s="2">
-        <v>108</v>
-      </c>
       <c r="F16" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>99</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17">
@@ -3143,28 +3258,28 @@
         <v>19</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="E17" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="E17" t="s" s="2">
-        <v>114</v>
-      </c>
       <c r="F17" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I17" t="s" s="2">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="J17" t="s" s="2">
         <v>119</v>
@@ -3172,39 +3287,39 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="B18" t="s" s="2">
+      <c r="C18" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="C18" t="s" s="2">
+      <c r="D18" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="D18" t="s" s="2">
+      <c r="E18" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="F18" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="E18" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="F18" t="s" s="2">
+      <c r="G18" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="G18" t="s" s="2">
+      <c r="H18" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="H18" t="s" s="2">
-        <v>52</v>
-      </c>
       <c r="I18" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="J18" t="s" s="2">
         <v>126</v>
-      </c>
-      <c r="J18" t="s" s="2">
-        <v>127</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>19</v>
+        <v>127</v>
       </c>
       <c r="B19" t="s" s="2">
         <v>128</v>
@@ -3225,7 +3340,7 @@
         <v>132</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>133</v>
@@ -3263,7 +3378,7 @@
         <v>140</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21">
@@ -3271,31 +3386,31 @@
         <v>19</v>
       </c>
       <c r="B21" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="C21" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="D21" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="E21" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="F21" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="G21" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="H21" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="J21" t="s" s="2">
         <v>141</v>
-      </c>
-      <c r="C21" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="D21" t="s" s="2">
-        <v>143</v>
-      </c>
-      <c r="E21" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="F21" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="G21" t="s" s="2">
-        <v>145</v>
-      </c>
-      <c r="H21" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I21" t="s" s="2">
-        <v>146</v>
-      </c>
-      <c r="J21" t="s" s="2">
-        <v>147</v>
       </c>
     </row>
     <row r="22">
@@ -3513,7 +3628,7 @@
         <v>194</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>195</v>
@@ -3524,39 +3639,39 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>197</v>
       </c>
-      <c r="B29" t="s" s="2">
+      <c r="C29" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="C29" t="s" s="2">
+      <c r="D29" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="D29" t="s" s="2">
+      <c r="E29" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="F29" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="E29" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="F29" t="s" s="2">
+      <c r="G29" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="G29" t="s" s="2">
+      <c r="H29" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I29" t="s" s="2">
         <v>202</v>
       </c>
-      <c r="H29" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I29" t="s" s="2">
+      <c r="J29" t="s" s="2">
         <v>203</v>
-      </c>
-      <c r="J29" t="s" s="2">
-        <v>204</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>19</v>
+        <v>204</v>
       </c>
       <c r="B30" t="s" s="2">
         <v>205</v>
@@ -3609,7 +3724,7 @@
         <v>216</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>217</v>
@@ -3641,7 +3756,7 @@
         <v>223</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>224</v>
@@ -3737,13 +3852,13 @@
         <v>244</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I35" t="s" s="2">
-        <v>160</v>
+        <v>245</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36">
@@ -3751,36 +3866,36 @@
         <v>19</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D36" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="E36" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="E36" t="s" s="2">
-        <v>247</v>
-      </c>
       <c r="F36" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I36" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>253</v>
+        <v>19</v>
       </c>
       <c r="B37" t="s" s="2">
         <v>254</v>
@@ -3804,42 +3919,42 @@
         <v>16</v>
       </c>
       <c r="I37" t="s" s="2">
-        <v>203</v>
+        <v>259</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>204</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>19</v>
+        <v>261</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D38" t="s" s="2">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E38" t="s" s="2">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F38" t="s" s="2">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I38" t="s" s="2">
-        <v>264</v>
+        <v>210</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>265</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39">
@@ -3847,31 +3962,31 @@
         <v>19</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D39" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="E39" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="E39" t="s" s="2">
-        <v>267</v>
-      </c>
       <c r="F39" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I39" t="s" s="2">
-        <v>231</v>
+        <v>272</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40">
@@ -3879,31 +3994,31 @@
         <v>19</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D40" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E40" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F40" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I40" t="s" s="2">
-        <v>160</v>
+        <v>279</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="41">
@@ -3911,31 +4026,31 @@
         <v>19</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D41" t="s" s="2">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E41" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F41" t="s" s="2">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>283</v>
+        <v>238</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>232</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42">
@@ -3943,31 +4058,31 @@
         <v>19</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D42" t="s" s="2">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E42" t="s" s="2">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F42" t="s" s="2">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I42" t="s" s="2">
-        <v>238</v>
+        <v>167</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43">
@@ -3975,31 +4090,31 @@
         <v>19</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C43" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D43" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E43" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F43" t="s" s="2">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H43" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>218</v>
+        <v>239</v>
       </c>
     </row>
     <row r="44">
@@ -4007,31 +4122,31 @@
         <v>19</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D44" t="s" s="2">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E44" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F44" t="s" s="2">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I44" t="s" s="2">
-        <v>301</v>
+        <v>245</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="45">
@@ -4039,36 +4154,36 @@
         <v>19</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C45" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D45" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E45" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F45" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H45" t="s" s="2">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>309</v>
+        <v>225</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>310</v>
+        <v>19</v>
       </c>
       <c r="B46" t="s" s="2">
         <v>311</v>
@@ -4121,7 +4236,7 @@
         <v>322</v>
       </c>
       <c r="H47" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I47" t="s" s="2">
         <v>323</v>
@@ -4153,10 +4268,10 @@
         <v>329</v>
       </c>
       <c r="H48" t="s" s="2">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I48" t="s" s="2">
-        <v>160</v>
+        <v>272</v>
       </c>
       <c r="J48" t="s" s="2">
         <v>330</v>
@@ -4164,34 +4279,34 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D49" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="E49" t="s" s="2">
         <v>333</v>
       </c>
-      <c r="E49" t="s" s="2">
-        <v>332</v>
-      </c>
       <c r="F49" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I49" t="s" s="2">
-        <v>224</v>
+        <v>337</v>
       </c>
       <c r="J49" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="50">
@@ -4199,31 +4314,31 @@
         <v>19</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D50" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E50" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F50" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I50" t="s" s="2">
-        <v>283</v>
+        <v>344</v>
       </c>
       <c r="J50" t="s" s="2">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="51">
@@ -4231,63 +4346,63 @@
         <v>19</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C51" t="s" s="2">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D51" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E51" t="s" s="2">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F51" t="s" s="2">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="H51" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I51" t="s" s="2">
-        <v>301</v>
+        <v>167</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>349</v>
+        <v>19</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C52" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D52" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E52" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="F52" t="s" s="2">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I52" t="s" s="2">
-        <v>355</v>
+        <v>231</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="53">
@@ -4295,28 +4410,28 @@
         <v>19</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C53" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D53" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="E53" t="s" s="2">
         <v>359</v>
       </c>
-      <c r="E53" t="s" s="2">
-        <v>358</v>
-      </c>
       <c r="F53" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I53" t="s" s="2">
-        <v>362</v>
+        <v>298</v>
       </c>
       <c r="J53" t="s" s="2">
         <v>363</v>
@@ -4348,7 +4463,7 @@
         <v>16</v>
       </c>
       <c r="I54" t="s" s="2">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="J54" t="s" s="2">
         <v>369</v>
@@ -4356,34 +4471,34 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>19</v>
+        <v>370</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C55" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D55" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="E55" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="E55" t="s" s="2">
-        <v>371</v>
-      </c>
       <c r="F55" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I55" t="s" s="2">
-        <v>160</v>
+        <v>376</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="56">
@@ -4391,31 +4506,31 @@
         <v>19</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C56" t="s" s="2">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D56" t="s" s="2">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E56" t="s" s="2">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F56" t="s" s="2">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I56" t="s" s="2">
-        <v>301</v>
+        <v>383</v>
       </c>
       <c r="J56" t="s" s="2">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="57">
@@ -4423,31 +4538,31 @@
         <v>19</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C57" t="s" s="2">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="D57" t="s" s="2">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E57" t="s" s="2">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="F57" t="s" s="2">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I57" t="s" s="2">
-        <v>387</v>
+        <v>316</v>
       </c>
       <c r="J57" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="58">
@@ -4455,31 +4570,31 @@
         <v>19</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D58" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E58" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F58" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="H58" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I58" t="s" s="2">
-        <v>301</v>
+        <v>167</v>
       </c>
       <c r="J58" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="59">
@@ -4487,36 +4602,36 @@
         <v>19</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C59" t="s" s="2">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D59" t="s" s="2">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E59" t="s" s="2">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F59" t="s" s="2">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="H59" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I59" t="s" s="2">
-        <v>400</v>
+        <v>316</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>402</v>
+        <v>19</v>
       </c>
       <c r="B60" t="s" s="2">
         <v>403</v>
@@ -4572,10 +4687,10 @@
         <v>16</v>
       </c>
       <c r="I61" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="J61" t="s" s="2">
         <v>415</v>
-      </c>
-      <c r="J61" t="s" s="2">
-        <v>416</v>
       </c>
     </row>
     <row r="62">
@@ -4583,36 +4698,36 @@
         <v>19</v>
       </c>
       <c r="B62" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="C62" t="s" s="2">
         <v>417</v>
       </c>
-      <c r="C62" t="s" s="2">
+      <c r="D62" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="D62" t="s" s="2">
+      <c r="E62" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="F62" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="E62" t="s" s="2">
-        <v>418</v>
-      </c>
-      <c r="F62" t="s" s="2">
+      <c r="G62" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="G62" t="s" s="2">
+      <c r="H62" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I62" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="H62" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I62" t="s" s="2">
+      <c r="J62" t="s" s="2">
         <v>422</v>
-      </c>
-      <c r="J62" t="s" s="2">
-        <v>423</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>19</v>
+        <v>423</v>
       </c>
       <c r="B63" t="s" s="2">
         <v>424</v>
@@ -4700,10 +4815,10 @@
         <v>16</v>
       </c>
       <c r="I65" t="s" s="2">
-        <v>415</v>
+        <v>443</v>
       </c>
       <c r="J65" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="66">
@@ -4711,31 +4826,31 @@
         <v>19</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C66" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D66" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="E66" t="s" s="2">
         <v>446</v>
       </c>
-      <c r="E66" t="s" s="2">
-        <v>445</v>
-      </c>
       <c r="F66" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="H66" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I66" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J66" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="67">
@@ -4743,31 +4858,31 @@
         <v>19</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C67" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D67" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="E67" t="s" s="2">
         <v>453</v>
       </c>
-      <c r="E67" t="s" s="2">
-        <v>452</v>
-      </c>
       <c r="F67" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G67" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="H67" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I67" t="s" s="2">
-        <v>429</v>
+        <v>457</v>
       </c>
       <c r="J67" t="s" s="2">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="68">
@@ -4775,31 +4890,31 @@
         <v>19</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C68" t="s" s="2">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="D68" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E68" t="s" s="2">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F68" t="s" s="2">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="H68" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I68" t="s" s="2">
-        <v>462</v>
+        <v>436</v>
       </c>
       <c r="J68" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="69">
@@ -4807,25 +4922,25 @@
         <v>19</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C69" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D69" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="E69" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="E69" t="s" s="2">
-        <v>465</v>
-      </c>
       <c r="F69" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G69" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="H69" t="s" s="2">
-        <v>469</v>
+        <v>16</v>
       </c>
       <c r="I69" t="s" s="2">
         <v>470</v>
@@ -4836,34 +4951,34 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B70" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="B70" t="s" s="2">
+      <c r="C70" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="C70" t="s" s="2">
+      <c r="D70" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="D70" t="s" s="2">
+      <c r="E70" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="F70" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="E70" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="F70" t="s" s="2">
+      <c r="G70" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="G70" t="s" s="2">
+      <c r="H70" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I70" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="J70" t="s" s="2">
         <v>477</v>
-      </c>
-      <c r="H70" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I70" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="J70" t="s" s="2">
-        <v>479</v>
       </c>
     </row>
     <row r="71">
@@ -4871,31 +4986,31 @@
         <v>19</v>
       </c>
       <c r="B71" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="C71" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="D71" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="C71" t="s" s="2">
+      <c r="E71" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="F71" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="D71" t="s" s="2">
+      <c r="G71" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="E71" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="F71" t="s" s="2">
+      <c r="H71" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I71" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="G71" t="s" s="2">
+      <c r="J71" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="H71" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I71" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="J71" t="s" s="2">
-        <v>486</v>
       </c>
     </row>
     <row r="72">
@@ -4903,63 +5018,63 @@
         <v>19</v>
       </c>
       <c r="B72" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="C72" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="D72" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="C72" t="s" s="2">
+      <c r="E72" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="F72" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="D72" t="s" s="2">
+      <c r="G72" t="s" s="2">
         <v>489</v>
       </c>
-      <c r="E72" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="F72" t="s" s="2">
+      <c r="H72" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="G72" t="s" s="2">
+      <c r="I72" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="H72" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I72" t="s" s="2">
-        <v>264</v>
-      </c>
       <c r="J72" t="s" s="2">
-        <v>265</v>
+        <v>492</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>19</v>
+        <v>493</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C73" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D73" t="s" s="2">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E73" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="F73" t="s" s="2">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I73" t="s" s="2">
-        <v>283</v>
+        <v>499</v>
       </c>
       <c r="J73" t="s" s="2">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="74">
@@ -4967,31 +5082,31 @@
         <v>19</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C74" t="s" s="2">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="D74" t="s" s="2">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="E74" t="s" s="2">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="F74" t="s" s="2">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I74" t="s" s="2">
-        <v>301</v>
+        <v>506</v>
       </c>
       <c r="J74" t="s" s="2">
-        <v>348</v>
+        <v>507</v>
       </c>
     </row>
     <row r="75">
@@ -4999,31 +5114,31 @@
         <v>19</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="C75" t="s" s="2">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D75" t="s" s="2">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="E75" t="s" s="2">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="F75" t="s" s="2">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="G75" t="s" s="2">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="H75" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I75" t="s" s="2">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="J75" t="s" s="2">
-        <v>509</v>
+        <v>514</v>
       </c>
     </row>
     <row r="76">
@@ -5031,63 +5146,63 @@
         <v>19</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="C76" t="s" s="2">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="D76" t="s" s="2">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="E76" t="s" s="2">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="F76" t="s" s="2">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="G76" t="s" s="2">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="H76" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I76" t="s" s="2">
-        <v>515</v>
+        <v>279</v>
       </c>
       <c r="J76" t="s" s="2">
-        <v>516</v>
+        <v>280</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>517</v>
+        <v>19</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="C77" t="s" s="2">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D77" t="s" s="2">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="E77" t="s" s="2">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F77" t="s" s="2">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="G77" t="s" s="2">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="H77" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I77" t="s" s="2">
-        <v>387</v>
+        <v>298</v>
       </c>
       <c r="J77" t="s" s="2">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="78">
@@ -5095,31 +5210,31 @@
         <v>19</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C78" t="s" s="2">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D78" t="s" s="2">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E78" t="s" s="2">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F78" t="s" s="2">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="G78" t="s" s="2">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="H78" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I78" t="s" s="2">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="J78" t="s" s="2">
-        <v>232</v>
+        <v>369</v>
       </c>
     </row>
     <row r="79">
@@ -5127,31 +5242,31 @@
         <v>19</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C79" t="s" s="2">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D79" t="s" s="2">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E79" t="s" s="2">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F79" t="s" s="2">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="G79" t="s" s="2">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="H79" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I79" t="s" s="2">
-        <v>301</v>
+        <v>536</v>
       </c>
       <c r="J79" t="s" s="2">
-        <v>348</v>
+        <v>537</v>
       </c>
     </row>
     <row r="80">
@@ -5159,63 +5274,63 @@
         <v>19</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="C80" t="s" s="2">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="D80" t="s" s="2">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="E80" t="s" s="2">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="F80" t="s" s="2">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="G80" t="s" s="2">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="H80" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I80" t="s" s="2">
-        <v>301</v>
+        <v>543</v>
       </c>
       <c r="J80" t="s" s="2">
-        <v>271</v>
+        <v>544</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>19</v>
+        <v>545</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="C81" t="s" s="2">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="D81" t="s" s="2">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="E81" t="s" s="2">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="F81" t="s" s="2">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="G81" t="s" s="2">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="H81" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I81" t="s" s="2">
-        <v>544</v>
+        <v>408</v>
       </c>
       <c r="J81" t="s" s="2">
-        <v>545</v>
+        <v>551</v>
       </c>
     </row>
     <row r="82">
@@ -5223,31 +5338,31 @@
         <v>19</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C82" t="s" s="2">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="D82" t="s" s="2">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E82" t="s" s="2">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="F82" t="s" s="2">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="G82" t="s" s="2">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="H82" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I82" t="s" s="2">
-        <v>264</v>
+        <v>316</v>
       </c>
       <c r="J82" t="s" s="2">
-        <v>551</v>
+        <v>239</v>
       </c>
     </row>
     <row r="83">
@@ -5255,31 +5370,31 @@
         <v>19</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="C83" t="s" s="2">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="D83" t="s" s="2">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="E83" t="s" s="2">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="F83" t="s" s="2">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="G83" t="s" s="2">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="H83" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I83" t="s" s="2">
-        <v>557</v>
+        <v>316</v>
       </c>
       <c r="J83" t="s" s="2">
-        <v>558</v>
+        <v>369</v>
       </c>
     </row>
     <row r="84">
@@ -5287,31 +5402,31 @@
         <v>19</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="C84" t="s" s="2">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="D84" t="s" s="2">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="E84" t="s" s="2">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="F84" t="s" s="2">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="G84" t="s" s="2">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="H84" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I84" t="s" s="2">
-        <v>557</v>
+        <v>316</v>
       </c>
       <c r="J84" t="s" s="2">
-        <v>564</v>
+        <v>286</v>
       </c>
     </row>
     <row r="85">
@@ -5319,31 +5434,31 @@
         <v>19</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="C85" t="s" s="2">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D85" t="s" s="2">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="E85" t="s" s="2">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="F85" t="s" s="2">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="G85" t="s" s="2">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="H85" t="s" s="2">
-        <v>52</v>
+        <v>125</v>
       </c>
       <c r="I85" t="s" s="2">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="J85" t="s" s="2">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="86">
@@ -5351,31 +5466,31 @@
         <v>19</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C86" t="s" s="2">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="D86" t="s" s="2">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="E86" t="s" s="2">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="F86" t="s" s="2">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="G86" t="s" s="2">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="H86" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I86" t="s" s="2">
-        <v>577</v>
+        <v>279</v>
       </c>
       <c r="J86" t="s" s="2">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="87">
@@ -5383,36 +5498,36 @@
         <v>19</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C87" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D87" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="E87" t="s" s="2">
         <v>581</v>
       </c>
-      <c r="E87" t="s" s="2">
-        <v>580</v>
-      </c>
       <c r="F87" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G87" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H87" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I87" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="J87" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>586</v>
+        <v>19</v>
       </c>
       <c r="B88" t="s" s="2">
         <v>587</v>
@@ -5436,10 +5551,10 @@
         <v>16</v>
       </c>
       <c r="I88" t="s" s="2">
+        <v>585</v>
+      </c>
+      <c r="J88" t="s" s="2">
         <v>592</v>
-      </c>
-      <c r="J88" t="s" s="2">
-        <v>593</v>
       </c>
     </row>
     <row r="89">
@@ -5447,31 +5562,31 @@
         <v>19</v>
       </c>
       <c r="B89" t="s" s="2">
+        <v>593</v>
+      </c>
+      <c r="C89" t="s" s="2">
         <v>594</v>
       </c>
-      <c r="C89" t="s" s="2">
+      <c r="D89" t="s" s="2">
         <v>595</v>
       </c>
-      <c r="D89" t="s" s="2">
+      <c r="E89" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="F89" t="s" s="2">
         <v>596</v>
       </c>
-      <c r="E89" t="s" s="2">
-        <v>595</v>
-      </c>
-      <c r="F89" t="s" s="2">
+      <c r="G89" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="G89" t="s" s="2">
+      <c r="H89" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I89" t="s" s="2">
         <v>598</v>
       </c>
-      <c r="H89" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="I89" t="s" s="2">
+      <c r="J89" t="s" s="2">
         <v>599</v>
-      </c>
-      <c r="J89" t="s" s="2">
-        <v>471</v>
       </c>
     </row>
     <row r="90">
@@ -5497,7 +5612,7 @@
         <v>604</v>
       </c>
       <c r="H90" t="s" s="2">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I90" t="s" s="2">
         <v>605</v>
@@ -5529,45 +5644,45 @@
         <v>611</v>
       </c>
       <c r="H91" t="s" s="2">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I91" t="s" s="2">
-        <v>577</v>
+        <v>612</v>
       </c>
       <c r="J91" t="s" s="2">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C92" t="s" s="2">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D92" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="E92" t="s" s="2">
         <v>616</v>
       </c>
-      <c r="E92" t="s" s="2">
-        <v>615</v>
-      </c>
       <c r="F92" t="s" s="2">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G92" t="s" s="2">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="H92" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I92" t="s" s="2">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="J92" t="s" s="2">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="93">
@@ -5575,31 +5690,31 @@
         <v>19</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C93" t="s" s="2">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D93" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="E93" t="s" s="2">
         <v>623</v>
       </c>
-      <c r="E93" t="s" s="2">
-        <v>622</v>
-      </c>
       <c r="F93" t="s" s="2">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="G93" t="s" s="2">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="H93" t="s" s="2">
-        <v>16</v>
+        <v>490</v>
       </c>
       <c r="I93" t="s" s="2">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="J93" t="s" s="2">
-        <v>627</v>
+        <v>492</v>
       </c>
     </row>
     <row r="94">
@@ -5625,13 +5740,13 @@
         <v>632</v>
       </c>
       <c r="H94" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I94" t="s" s="2">
         <v>633</v>
       </c>
       <c r="J94" t="s" s="2">
-        <v>627</v>
+        <v>634</v>
       </c>
     </row>
     <row r="95">
@@ -5639,28 +5754,28 @@
         <v>19</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="C95" t="s" s="2">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D95" t="s" s="2">
+        <v>637</v>
+      </c>
+      <c r="E95" t="s" s="2">
         <v>636</v>
       </c>
-      <c r="E95" t="s" s="2">
-        <v>635</v>
-      </c>
       <c r="F95" t="s" s="2">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="H95" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I95" t="s" s="2">
-        <v>639</v>
+        <v>605</v>
       </c>
       <c r="J95" t="s" s="2">
         <v>640</v>
@@ -5668,34 +5783,34 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>19</v>
+        <v>641</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C96" t="s" s="2">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D96" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="E96" t="s" s="2">
         <v>643</v>
       </c>
-      <c r="E96" t="s" s="2">
-        <v>642</v>
-      </c>
       <c r="F96" t="s" s="2">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G96" t="s" s="2">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="H96" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I96" t="s" s="2">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="97">
@@ -5703,31 +5818,31 @@
         <v>19</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C97" t="s" s="2">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="D97" t="s" s="2">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="E97" t="s" s="2">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="F97" t="s" s="2">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="G97" t="s" s="2">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="H97" t="s" s="2">
         <v>16</v>
       </c>
       <c r="I97" t="s" s="2">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="J97" t="s" s="2">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="98">
@@ -5735,31 +5850,31 @@
         <v>19</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="C98" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="D98" t="s" s="2">
+        <v>658</v>
+      </c>
+      <c r="E98" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="F98" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="G98" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="H98" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I98" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="J98" t="s" s="2">
         <v>655</v>
-      </c>
-      <c r="D98" t="s" s="2">
-        <v>656</v>
-      </c>
-      <c r="E98" t="s" s="2">
-        <v>655</v>
-      </c>
-      <c r="F98" t="s" s="2">
-        <v>657</v>
-      </c>
-      <c r="G98" t="s" s="2">
-        <v>658</v>
-      </c>
-      <c r="H98" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I98" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="J98" t="s" s="2">
-        <v>660</v>
       </c>
     </row>
     <row r="99">
@@ -5767,36 +5882,36 @@
         <v>19</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C99" t="s" s="2">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D99" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="E99" t="s" s="2">
         <v>663</v>
       </c>
-      <c r="E99" t="s" s="2">
-        <v>662</v>
-      </c>
       <c r="F99" t="s" s="2">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="H99" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I99" t="s" s="2">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="J99" t="s" s="2">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>668</v>
+        <v>19</v>
       </c>
       <c r="B100" t="s" s="2">
         <v>669</v>
@@ -5817,13 +5932,13 @@
         <v>673</v>
       </c>
       <c r="H100" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I100" t="s" s="2">
+        <v>667</v>
+      </c>
+      <c r="J100" t="s" s="2">
         <v>674</v>
-      </c>
-      <c r="J100" t="s" s="2">
-        <v>675</v>
       </c>
     </row>
     <row r="101">
@@ -5831,31 +5946,31 @@
         <v>19</v>
       </c>
       <c r="B101" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="C101" t="s" s="2">
         <v>676</v>
       </c>
-      <c r="C101" t="s" s="2">
+      <c r="D101" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="D101" t="s" s="2">
+      <c r="E101" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="F101" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="E101" t="s" s="2">
-        <v>677</v>
-      </c>
-      <c r="F101" t="s" s="2">
+      <c r="G101" t="s" s="2">
         <v>679</v>
       </c>
-      <c r="G101" t="s" s="2">
+      <c r="H101" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I101" t="s" s="2">
         <v>680</v>
       </c>
-      <c r="H101" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I101" t="s" s="2">
+      <c r="J101" t="s" s="2">
         <v>681</v>
-      </c>
-      <c r="J101" t="s" s="2">
-        <v>682</v>
       </c>
     </row>
     <row r="102">
@@ -5863,28 +5978,28 @@
         <v>19</v>
       </c>
       <c r="B102" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="C102" t="s" s="2">
         <v>683</v>
       </c>
-      <c r="C102" t="s" s="2">
+      <c r="D102" t="s" s="2">
         <v>684</v>
       </c>
-      <c r="D102" t="s" s="2">
+      <c r="E102" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="F102" t="s" s="2">
         <v>685</v>
       </c>
-      <c r="E102" t="s" s="2">
-        <v>684</v>
-      </c>
-      <c r="F102" t="s" s="2">
+      <c r="G102" t="s" s="2">
         <v>686</v>
       </c>
-      <c r="G102" t="s" s="2">
+      <c r="H102" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I102" t="s" s="2">
         <v>687</v>
-      </c>
-      <c r="H102" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I102" t="s" s="2">
-        <v>674</v>
       </c>
       <c r="J102" t="s" s="2">
         <v>688</v>
@@ -5913,7 +6028,7 @@
         <v>693</v>
       </c>
       <c r="H103" t="s" s="2">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I103" t="s" s="2">
         <v>694</v>
@@ -5924,34 +6039,34 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>19</v>
+        <v>696</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C104" t="s" s="2">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="D104" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="E104" t="s" s="2">
         <v>698</v>
       </c>
-      <c r="E104" t="s" s="2">
-        <v>697</v>
-      </c>
       <c r="F104" t="s" s="2">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="G104" t="s" s="2">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="H104" t="s" s="2">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="I104" t="s" s="2">
-        <v>674</v>
+        <v>702</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="105">
@@ -5959,31 +6074,31 @@
         <v>19</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="C105" t="s" s="2">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="D105" t="s" s="2">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="E105" t="s" s="2">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="F105" t="s" s="2">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="G105" t="s" s="2">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="H105" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I105" t="s" s="2">
-        <v>674</v>
+        <v>709</v>
       </c>
       <c r="J105" t="s" s="2">
-        <v>707</v>
+        <v>710</v>
       </c>
     </row>
     <row r="106">
@@ -5991,31 +6106,31 @@
         <v>19</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="C106" t="s" s="2">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="D106" t="s" s="2">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="E106" t="s" s="2">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="F106" t="s" s="2">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="G106" t="s" s="2">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="H106" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I106" t="s" s="2">
-        <v>674</v>
+        <v>702</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>707</v>
+        <v>716</v>
       </c>
     </row>
     <row r="107">
@@ -6023,63 +6138,63 @@
         <v>19</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="C107" t="s" s="2">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="D107" t="s" s="2">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="E107" t="s" s="2">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="F107" t="s" s="2">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="G107" t="s" s="2">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="H107" t="s" s="2">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="I107" t="s" s="2">
-        <v>160</v>
+        <v>722</v>
       </c>
       <c r="J107" t="s" s="2">
-        <v>718</v>
+        <v>723</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>719</v>
+        <v>19</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="C108" t="s" s="2">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="D108" t="s" s="2">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="E108" t="s" s="2">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="F108" t="s" s="2">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="H108" t="s" s="2">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="I108" t="s" s="2">
-        <v>725</v>
+        <v>702</v>
       </c>
       <c r="J108" t="s" s="2">
-        <v>726</v>
+        <v>729</v>
       </c>
     </row>
     <row r="109">
@@ -6087,31 +6202,31 @@
         <v>19</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="C109" t="s" s="2">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="D109" t="s" s="2">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="E109" t="s" s="2">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="F109" t="s" s="2">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="H109" t="s" s="2">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="I109" t="s" s="2">
-        <v>725</v>
+        <v>702</v>
       </c>
       <c r="J109" t="s" s="2">
-        <v>726</v>
+        <v>735</v>
       </c>
     </row>
     <row r="110">
@@ -6119,31 +6234,31 @@
         <v>19</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="C110" t="s" s="2">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="D110" t="s" s="2">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="E110" t="s" s="2">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="F110" t="s" s="2">
+        <v>739</v>
+      </c>
+      <c r="G110" t="s" s="2">
+        <v>740</v>
+      </c>
+      <c r="H110" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="I110" t="s" s="2">
+        <v>702</v>
+      </c>
+      <c r="J110" t="s" s="2">
         <v>735</v>
-      </c>
-      <c r="G110" t="s" s="2">
-        <v>736</v>
-      </c>
-      <c r="H110" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="I110" t="s" s="2">
-        <v>737</v>
-      </c>
-      <c r="J110" t="s" s="2">
-        <v>726</v>
       </c>
     </row>
     <row r="111">
@@ -6151,31 +6266,159 @@
         <v>19</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="C111" t="s" s="2">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="D111" t="s" s="2">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="E111" t="s" s="2">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="F111" t="s" s="2">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="G111" t="s" s="2">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="H111" t="s" s="2">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="I111" t="s" s="2">
-        <v>544</v>
+        <v>167</v>
       </c>
       <c r="J111" t="s" s="2">
-        <v>726</v>
+        <v>746</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="B112" t="s" s="2">
+        <v>748</v>
+      </c>
+      <c r="C112" t="s" s="2">
+        <v>749</v>
+      </c>
+      <c r="D112" t="s" s="2">
+        <v>750</v>
+      </c>
+      <c r="E112" t="s" s="2">
+        <v>749</v>
+      </c>
+      <c r="F112" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="G112" t="s" s="2">
+        <v>752</v>
+      </c>
+      <c r="H112" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="I112" t="s" s="2">
+        <v>753</v>
+      </c>
+      <c r="J112" t="s" s="2">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B113" t="s" s="2">
+        <v>755</v>
+      </c>
+      <c r="C113" t="s" s="2">
+        <v>756</v>
+      </c>
+      <c r="D113" t="s" s="2">
+        <v>757</v>
+      </c>
+      <c r="E113" t="s" s="2">
+        <v>756</v>
+      </c>
+      <c r="F113" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="G113" t="s" s="2">
+        <v>759</v>
+      </c>
+      <c r="H113" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="I113" t="s" s="2">
+        <v>753</v>
+      </c>
+      <c r="J113" t="s" s="2">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B114" t="s" s="2">
+        <v>760</v>
+      </c>
+      <c r="C114" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="D114" t="s" s="2">
+        <v>762</v>
+      </c>
+      <c r="E114" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="F114" t="s" s="2">
+        <v>763</v>
+      </c>
+      <c r="G114" t="s" s="2">
+        <v>764</v>
+      </c>
+      <c r="H114" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="I114" t="s" s="2">
+        <v>765</v>
+      </c>
+      <c r="J114" t="s" s="2">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B115" t="s" s="2">
+        <v>766</v>
+      </c>
+      <c r="C115" t="s" s="2">
+        <v>767</v>
+      </c>
+      <c r="D115" t="s" s="2">
+        <v>768</v>
+      </c>
+      <c r="E115" t="s" s="2">
+        <v>767</v>
+      </c>
+      <c r="F115" t="s" s="2">
+        <v>769</v>
+      </c>
+      <c r="G115" t="s" s="2">
+        <v>770</v>
+      </c>
+      <c r="H115" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="I115" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="J115" t="s" s="2">
+        <v>754</v>
       </c>
     </row>
   </sheetData>
@@ -6187,18 +6430,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>743</v>
+        <v>771</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>744</v>
+        <v>772</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>745</v>
+        <v>773</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>746</v>
+        <v>774</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>19</v>
@@ -6212,10 +6455,10 @@
         <v>19</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>747</v>
+        <v>775</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>748</v>
+        <v>776</v>
       </c>
     </row>
     <row r="4">
@@ -6223,10 +6466,10 @@
         <v>19</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>749</v>
+        <v>777</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>750</v>
+        <v>778</v>
       </c>
     </row>
     <row r="5">
@@ -6234,10 +6477,10 @@
         <v>19</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>751</v>
+        <v>779</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>752</v>
+        <v>780</v>
       </c>
     </row>
     <row r="6">
@@ -6245,10 +6488,10 @@
         <v>19</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>753</v>
+        <v>781</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>754</v>
+        <v>782</v>
       </c>
     </row>
     <row r="7">
@@ -6256,10 +6499,10 @@
         <v>19</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>218</v>
+        <v>783</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>755</v>
+        <v>784</v>
       </c>
     </row>
     <row r="8">
@@ -6267,10 +6510,10 @@
         <v>19</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>756</v>
+        <v>785</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>757</v>
+        <v>786</v>
       </c>
     </row>
     <row r="9">
@@ -6278,10 +6521,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>758</v>
+        <v>787</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>759</v>
+        <v>788</v>
       </c>
     </row>
     <row r="10">
@@ -6289,10 +6532,10 @@
         <v>19</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>760</v>
+        <v>225</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>761</v>
+        <v>789</v>
       </c>
     </row>
     <row r="11">
@@ -6300,10 +6543,10 @@
         <v>19</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>762</v>
+        <v>790</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>763</v>
+        <v>791</v>
       </c>
     </row>
     <row r="12">
@@ -6311,10 +6554,10 @@
         <v>19</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>764</v>
+        <v>792</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>765</v>
+        <v>793</v>
       </c>
     </row>
     <row r="13">
@@ -6322,10 +6565,10 @@
         <v>19</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>225</v>
+        <v>794</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>766</v>
+        <v>795</v>
       </c>
     </row>
     <row r="14">
@@ -6333,10 +6576,10 @@
         <v>19</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>767</v>
+        <v>796</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>768</v>
+        <v>797</v>
       </c>
     </row>
     <row r="15">
@@ -6344,10 +6587,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>769</v>
+        <v>798</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>770</v>
+        <v>799</v>
       </c>
     </row>
     <row r="16">
@@ -6355,10 +6598,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>771</v>
+        <v>232</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>772</v>
+        <v>800</v>
       </c>
     </row>
     <row r="17">
@@ -6366,10 +6609,10 @@
         <v>19</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>773</v>
+        <v>801</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>774</v>
+        <v>802</v>
       </c>
     </row>
     <row r="18">
@@ -6377,10 +6620,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>134</v>
+        <v>803</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>775</v>
+        <v>804</v>
       </c>
     </row>
     <row r="19">
@@ -6388,10 +6631,10 @@
         <v>19</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>189</v>
+        <v>805</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>776</v>
+        <v>806</v>
       </c>
     </row>
     <row r="20">
@@ -6399,10 +6642,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>516</v>
+        <v>807</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>777</v>
+        <v>808</v>
       </c>
     </row>
     <row r="21">
@@ -6410,10 +6653,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>778</v>
+        <v>809</v>
       </c>
     </row>
     <row r="22">
@@ -6421,10 +6664,10 @@
         <v>19</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>779</v>
+        <v>196</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>780</v>
+        <v>810</v>
       </c>
     </row>
     <row r="23">
@@ -6432,10 +6675,10 @@
         <v>19</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>781</v>
+        <v>544</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>782</v>
+        <v>811</v>
       </c>
     </row>
     <row r="24">
@@ -6443,10 +6686,10 @@
         <v>19</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>783</v>
+        <v>812</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>784</v>
+        <v>813</v>
       </c>
     </row>
     <row r="25">
@@ -6454,10 +6697,10 @@
         <v>19</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>785</v>
+        <v>814</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>786</v>
+        <v>815</v>
       </c>
     </row>
     <row r="26">
@@ -6465,10 +6708,10 @@
         <v>19</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>787</v>
+        <v>816</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>788</v>
+        <v>817</v>
       </c>
     </row>
     <row r="27">
@@ -6476,10 +6719,10 @@
         <v>19</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>558</v>
+        <v>818</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>789</v>
+        <v>819</v>
       </c>
     </row>
     <row r="28">
@@ -6487,21 +6730,21 @@
         <v>19</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>19</v>
+        <v>820</v>
       </c>
       <c r="C28" t="s" s="2">
-        <v>19</v>
+        <v>821</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>790</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>19</v>
+        <v>822</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>19</v>
+        <v>823</v>
       </c>
     </row>
     <row r="30">
@@ -6509,10 +6752,10 @@
         <v>19</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>791</v>
+        <v>586</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>792</v>
+        <v>824</v>
       </c>
     </row>
     <row r="31">
@@ -6520,21 +6763,21 @@
         <v>19</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>793</v>
+        <v>19</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>794</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>19</v>
+        <v>825</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>795</v>
+        <v>19</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>796</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33">
@@ -6542,10 +6785,10 @@
         <v>19</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>797</v>
+        <v>826</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>798</v>
+        <v>827</v>
       </c>
     </row>
     <row r="34">
@@ -6553,10 +6796,10 @@
         <v>19</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>799</v>
+        <v>828</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>800</v>
+        <v>829</v>
       </c>
     </row>
     <row r="35">
@@ -6564,10 +6807,10 @@
         <v>19</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>801</v>
+        <v>830</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>802</v>
+        <v>831</v>
       </c>
     </row>
     <row r="36">
@@ -6575,10 +6818,10 @@
         <v>19</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>803</v>
+        <v>832</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>804</v>
+        <v>833</v>
       </c>
     </row>
     <row r="37">
@@ -6586,10 +6829,10 @@
         <v>19</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>805</v>
+        <v>834</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>806</v>
+        <v>835</v>
       </c>
     </row>
     <row r="38">
@@ -6597,10 +6840,10 @@
         <v>19</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>807</v>
+        <v>836</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>808</v>
+        <v>837</v>
       </c>
     </row>
     <row r="39">
@@ -6608,10 +6851,54 @@
         <v>19</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>809</v>
+        <v>838</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>810</v>
+        <v>839</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>840</v>
+      </c>
+      <c r="C40" t="s" s="2">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>842</v>
+      </c>
+      <c r="C41" t="s" s="2">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>844</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>846</v>
+      </c>
+      <c r="C43" t="s" s="2">
+        <v>847</v>
       </c>
     </row>
   </sheetData>
@@ -6626,43 +6913,43 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>811</v>
+        <v>848</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>812</v>
+        <v>849</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>813</v>
+        <v>850</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>703</v>
+        <v>731</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>706</v>
+        <v>734</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>814</v>
+        <v>851</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>709</v>
+        <v>737</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>712</v>
+        <v>740</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>815</v>
+        <v>852</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>714</v>
+        <v>742</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>717</v>
+        <v>745</v>
       </c>
     </row>
   </sheetData>
@@ -6686,58 +6973,58 @@
         <v>4</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>816</v>
+        <v>853</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>702</v>
+        <v>730</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>668</v>
+        <v>696</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>704</v>
+        <v>732</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>703</v>
+        <v>731</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>707</v>
+        <v>735</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>708</v>
+        <v>736</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>668</v>
+        <v>696</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>710</v>
+        <v>738</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>709</v>
+        <v>737</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>707</v>
+        <v>735</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>713</v>
+        <v>741</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>668</v>
+        <v>696</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>715</v>
+        <v>743</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>714</v>
+        <v>742</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>718</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement flow-active error coverage
</commit_message>
<xml_diff>
--- a/docs/test_plan/I3C_Testplan.xlsx
+++ b/docs/test_plan/I3C_Testplan.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="891">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -849,7 +849,7 @@
 Stimulus / Actions: Queue first write (`toc=0`) and second write (`toc=1`) with distinct payloads; separately issue a `toc=0` write with no next supported command.</t>
   </si>
   <si>
-    <t xml:space="preserve">Valid case: first write completes data/T-bit then emits `Sr`; **data integrity check: for each transfer, `sampled_data[i]` matches its own TX FIFO byte slice** — confirming the RSTART boundary does not cause data loss, duplication, or cross-command mixing; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; both RESPs report success with matching TID/length. With broadcast-header enabled, only the first private transfer emits the `0x7e` preamble. Negative case: the first write data is transmitted, controller emits STOP instead of RSTART, and RESP is `Success` with actual length transmitted.</t>
+    <t xml:space="preserve">Valid case: first write completes data/T-bit then emits `Sr`; **data integrity check: for each transfer, `sampled_data[i]` matches its own TX FIFO byte slice** — confirming the RSTART boundary does not cause data loss, duplication, or cross-command mixing; second command starts after `Sr`; final STOP occurs only after the `toc=1` command; each `wroc=1` command reports success with matching TID/length. With broadcast-header enabled, only the first private transfer emits the `0x7e` preamble. Negative case: the first write data is transmitted, controller emits STOP instead of RSTART, and RESP is `NotSupported` with actual length transmitted regardless of WROC.</t>
   </si>
   <si>
     <t xml:space="preserve">`flow_active`, `scl_generator`, UVM scoreboard</t>
@@ -1063,10 +1063,10 @@
 Stimulus / Actions: Sweep `dtt` 0..7 in both private-address modes (no broadcast header and with broadcast header).</t>
   </si>
   <si>
-    <t xml:space="preserve">**`dtt` 0..4 (positive):** the correct number of inline bytes is transmitted; **data integrity check: `sampled_data[i]` == cmd byte i for i &lt; dtt** — confirming the cmd dword bytes are sent in descriptor order with no extra, missing, or reordered byte; RESP `Success`; `resp.length == dtt`. **`dtt` 5..7 (negative):** FSM rejects in `WaitDAT` before any bus activity; `not_supported_d` is set; RESP error is `NotSupported` (4'hA); no inline bytes sent, queues remain clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active` (`WaitDAT` early-exit), CMD descriptor</t>
+    <t xml:space="preserve">**`dtt` 0..4 (positive):** the correct number of inline bytes is transmitted; **data integrity check: `sampled_data[i]` == cmd byte i for i &lt; dtt** — confirming the cmd dword bytes are sent in descriptor order with no extra, missing, or reordered byte; RESP `Success`; `resp.length == dtt`. **`dtt` 5..7 (negative):** FSM rejects in `FetchDAT` before DAT or bus activity; `not_supported_d` is set; RESP error is `NotSupported` (4'hA); no inline bytes sent, queues remain clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active` (`FetchDAT` validation), CMD descriptor</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_imm_dtt`, `cp_resp_err`, `cp_private_start_prefix`</t>
@@ -1082,7 +1082,7 @@
   </si>
   <si>
     <t xml:space="preserve">Preconditions: DAT[0] I3C device; target ACKs address and data; `dtt=2`, bytes `[AA, BB]`.
-Stimulus / Actions: Issue one immediate command with `toc=1` and one with `toc=0`; cover both I3C and I2C immediate paths (`I3CWriteImmediate`, `I2CWriteImmediate`).</t>
+Stimulus / Actions: Issue one immediate command with `toc=1` and one with `toc=0`; cover both private I3C and I2C immediate paths through `InitI3CWrite`/`InitI2CWrite` and `IssueCmd`.</t>
   </si>
   <si>
     <t xml:space="preserve">`toc=1`: STOP is generated after inline data; **data integrity check: `sampled_data[0]`==`0xAA`, `sampled_data[1]`==`0xBB`**; RESP is `Success` with correct length 2. `toc=0`: all dtt bytes are still transmitted before STOP — **data integrity check: same byte-level check applies**; STOP is generated, `not_supported_d` is set, RESP error is `NotSupported` (4'hA); no `Sr` or continuation occurs. Both toc values must complete all dtt bytes on bus with correct values before STOP. Bus must not hang.</t>
@@ -1474,23 +1474,20 @@
     <t xml:space="preserve">ERR_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify successful RESP descriptor fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`resp_success_tid_length`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: Valid transactions with unique TIDs.
-Stimulus / Actions: Run immediate, regular write, regular read, and ENTDAA success paths.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RESP `[31:28]=Success`, `[27:24]=TID`, `[15:0]=actual length`.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, RESP FIFO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_resp_err`, `cp_tid`, `cp_resp_len`</t>
+    <t xml:space="preserve">Verify successful RESP descriptor fields without a dedicated vseq.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: SVA enabled; immediate, regular write/read, I2C, CCC, and ENTDAA success paths are exercised by existing functional vseqs.
+Stimulus / Actions: No standalone stimulus. Existing success-path vseqs naturally produce successful responses; `flow_active_sva` checks the common Success/TID/reserved/length encoding at RESP write time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESP `[31:28]=Success`, `[27:24]=TID`, `[23:16]=0`, and `[15:0]=actual length` for every covered successful command class.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, RESP FIFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_sdr_write_toc1_success_resp`, `cp_sdr_read_success_resp_len`, `cp_i2c_write_success_resp`, `cp_i2c_read_success_resp`, `cp_imm_success_resp`, `cp_daa_success_resp`, CCC success RESP covers</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_002</t>
@@ -1509,26 +1506,26 @@
     <t xml:space="preserve">RESP status is `AddrHeader`, TID matches the command, reserved bits are zero, and length is 0 for every supported command class with private/target address NACK. No regular data, read data, immediate inline data, or direct CCC target data is transferred after the NACK.</t>
   </si>
   <si>
-    <t xml:space="preserve">`cp_resp_err`, `cp_addr_ack`, `cp_tid`, `cp_resp_len`, `cross_imm_x_device_type`</t>
+    <t xml:space="preserve">`cp_sdr_write_addr_nack_resp`, `cp_sdr_read_addr_nack_resp`, `cp_i2c_write_addr_nack_resp`, `cp_i2c_read_addr_nack_resp`, `cp_i3c_imm_addr_nack_resp`, `cp_i2c_imm_addr_nack_resp`, `cp_direct_ccc_target_addr_nack_resp`, `cp_addr_ack`, `cross_imm_x_device_type`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_003</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify `AddrHeader` response encoding and payload suppression when broadcast header `7'h7E+W` is NACKed.</t>
+    <t xml:space="preserve">Verify command-agnostic `AddrHeader` response encoding and follow-up suppression when the shared broadcast header `7'h7E+W` is NACKed.</t>
   </si>
   <si>
     <t xml:space="preserve">`resp_broadcast_header_nack`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Device NACKs `7'h7E+W` during a CCC command (ENEC/DISEC/ENTDAA).
-Stimulus / Actions: Run `i3c_broadcast_header_nack_resp_vseq`: issue ENEC, DISEC, and ENTDAA commands while the device NACKs the broadcast header.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RESP status is `AddrHeader`, TID matches the command, reserved bits are zero, and length is 0. No CCC opcode, CCC payload byte, or ENTDAA `7'h7E+R` round is emitted after the NACK; bus recovery is legal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_resp_err`, `cp_addr_ack`, `cp_tid`, `cp_resp_len`, `cp_ccc_nack`</t>
+    <t xml:space="preserve">Preconditions: Device NACKs `7'h7E+W` while the controller is in the common broadcast-header frame.
+Stimulus / Actions: Run `i3c_broadcast_header_nack_resp_vseq` to exercise a representative broadcast-header NACK; `flow_active_sva` checks the common `I3CBcastHeader` NACK path independent of whether the pending command is CCC, ENTDAA, or a private I3C transfer using the broadcast-header preamble.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESP status is `AddrHeader`, TID matches the command, reserved bits are zero, and length is 0. No command-specific follow-up is emitted after the NACK: no CCC opcode/payload, no ENTDAA `7'h7E+R` round, no private target-address phase, and no transfer data. Bus recovery is legal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_bcast_header_nack_sample_no_followup`, `cp_bcast_header_nack_stops_no_followup`, `cp_bcast_header_nack_resp`, `cp_addr_nack_resp`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_004</t>
@@ -1541,16 +1538,16 @@
   </si>
   <si>
     <t xml:space="preserve">Preconditions: Target ACKs the address and NACKs a data byte.
-Stimulus / Actions: Run `i2c_data_nack_write_vseq` with a multi-DWORD payload and `i3c_imm_data_nack_i2c_vseq` with `dtt=2..4`. Follow each error path with a successful transfer using the recovery policy appropriate to its data source.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The NACKed byte is fully clocked, but no later regular or inline byte is transmitted. Pre-NACK data matches the programmed TX FIFO or descriptor bytes. RESP is `Nack` with matching TID, zero reserved bits, and actual length through the NACKed byte. Regular write can preserve unfetched TX FIFO words, so recovery waits for idle and uses SW reset before the next FIFO-backed write. Immediate data is descriptor-resident, so its next transfer succeeds without SW reset.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `hci_queues`, `bus_tx_flow`, RESP FIFO, UVM scoreboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_data_ack`, `cp_resp_err`, `cp_tid`, `cp_resp_len`, `cross_imm_x_device_type`</t>
+Stimulus / Actions: Run `i2c_data_nack_write_vseq` with a multi-DWORD payload and first/middle/final data-byte NACK positions. Run `i3c_imm_data_nack_i2c_vseq` with `dtt=2..4`, covering first, middle, and final inline-byte NACK positions. Follow each error path with the recovery policy appropriate to its data source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The NACKed byte is fully clocked, but no later regular or inline byte is transmitted. Pre-NACK data matches the programmed TX FIFO or descriptor bytes. RESP is `I2cDataNackOrI3cBusAborted` with matching TID, zero reserved bits, and actual length through the NACKed byte. Regular write can preserve unfetched TX FIFO words, so recovery waits for idle and uses SW reset before the next FIFO-backed write. Immediate data is descriptor-resident, so its next transfer succeeds without SW reset.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `hci_queues`, `bus_tx_flow`, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_i2c_write_data_nack_latches`, `cp_i2c_write_data_nack_stops_no_more_data`, `cp_i2c_imm_data_nack_latches`, `cp_i2c_imm_data_nack_stops_no_more_data`, `cp_data_nack_resp`, `cp_i2c_write_data_nack_resp`, `cp_i2c_imm_data_nack_resp`, `cross_imm_x_device_type`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_005</t>
@@ -1563,120 +1560,123 @@
   </si>
   <si>
     <t xml:space="preserve">Preconditions: Target ends an I3C read after M bytes where M&lt;N requested bytes.
-Stimulus / Actions: Run `i3c_read_short_target_end_vseq` across multiple partial-DWORD boundaries and both private-address modes, including a `toc=0` command with a following command queued.</t>
+Stimulus / Actions: Run `i3c_read_short_target_end_vseq` across all partial-DWORD packing positions and both private-address modes, explicitly including the off-by-one boundary M=N-1 and a `toc=0` command with a following command queued.</t>
   </si>
   <si>
     <t xml:space="preserve">RX FIFO contains exactly the M valid bytes with correct packing; no fabricated byte is stored. Short read forces STOP and suppresses a requested continuation. RESP is `I3cShortReadErr` with matching TID, zero reserved bits, and actual length M. Draining RX and RESP data leaves queues ready for the next command; SW reset is not required.</t>
   </si>
   <si>
-    <t xml:space="preserve">`flow_active`, `bus_rx_flow`, RESP FIFO, UVM scoreboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_short_read`, `cp_resp_err`, `cp_tid`, `cp_resp_len`, `cp_private_start_prefix`</t>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `bus_rx_flow`, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_sdr_read_target_tbit_end_sets_short`, `cp_sdr_read_one_byte_short`, `cp_sdr_read_short_dword_boundary`, `cp_sdr_read_short_commits_received_word_and_stops`, `cp_sdr_read_short_blocks_more_data_and_continuation`, `cp_sdr_read_short_resp_len`, `cp_private_start_prefix`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_006</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify response classification and end-of-data handling for a legal SDR read final T-bit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`i3c_read_tbit_no_parity_resp`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: DAT[0] is I3C dynamic address `0x08`; target ends transfer with T-bit=0 at the requested length.
-Stimulus / Actions: Run `i3c_read_tbit_no_parity_resp_vseq` in both private-address modes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each mode uses the expected private-address prefix. Final T-bit=0 at the requested length is treated as legal end-of-data, no extra RX byte is consumed, queues drain cleanly, and the condition is not classified as `Parity`. RESP is `Success`, TID matches the command, reserved bits are zero, and length matches the requested length.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_read_tbit`, `cp_private_start_prefix`, `cp_resp_err`, `cp_tid`, `cp_resp_len`</t>
+    <t xml:space="preserve">Verify response classification and end-of-data handling for a legal SDR read final T-bit without a dedicated vseq.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: SVA enabled; existing SDR read vseqs drive final T-bit=0 at the requested length in both private-address modes.
+Stimulus / Actions: No standalone stimulus. `i3c_read_vseq` and `i3c_read_len_sweep_vseq` naturally exercise this condition; `flow_active_sva` checks the final T-bit transition and the resulting response.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final T-bit=0 at the requested length clears the remaining count without setting short-read state or consuming an extra RX byte. RESP is `Success`, TID matches the command, reserved bits are zero, and length matches the requested length, so the condition cannot be classified as `Parity`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `bus_rx_flow`, RESP FIFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_sdr_read_target_end_at_requested_len`, `cp_sdr_read_final_tbit_end_policy`, `cp_sdr_read_success_resp_len`, `cp_private_start_prefix`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_007</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify TX underflow/RX overflow termination, data boundary, response encoding, and recovery policy, including ENTDAA result storage overflow.</t>
+    <t xml:space="preserve">Verify I3C/I2C TX underflow and RX overflow termination, data boundary, response encoding, continuation suppression, and recovery, including ENTDAA result overflow.</t>
   </si>
   <si>
     <t xml:space="preserve">`resp_ovl_error`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: TX FIFO underflow, regular-read RX FIFO overflow, or ENTDAA result RX FIFO overflow condition.
-Stimulus / Actions: Run `i3c_ovl_resp_vseq`, `i3c_write_tx_fifo_underflow_vseq`, `i3c_read_rx_fifo_full_overflow_vseq`, and `i3c_entdaa_rx_fifo_partial_overflow_vseq`, including full/partial RX prefill, `toc=0/1`, both private-address modes, late TX refill, and ENTDAA result storage with only 0, 1, or 2 free RX FIFO entries for the 3-DWORD DAA result.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Committed TX/RX/DAA-result data remains correct and no garbage is emitted or stored. Overflow/underflow forces STOP and suppresses continuation. RESP is `Ovl` with matching TID, zero reserved bits, and the processed/committed boundary length. Regular-read RX overflow recovery drains preserved RX FIFO contents and RESP; no SW reset is required. ENTDAA result overflow drains the prefilled RX words plus any committed DAA result DWORDs and RESP; no SW reset is required. Residual/late TX data requires waiting for idle and issuing SW reset before a clean FIFO-backed recovery transfer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `hci_queues`, `scl_generator`, `entdaa_controller`, RX FIFO, RESP FIFO, UVM scoreboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_resp_err_ovl`, `cp_daa_result`, `cp_tid`, `cp_resp_len`, `cp_tx_empty`, `cp_tx_late_refill`, `cp_rx_full`, `cp_stall_type`</t>
+    <t xml:space="preserve">Preconditions: A regular I3C/I2C write exhausts TX FIFO, a regular I3C/I2C read cannot commit a full or partial DWORD to RX FIFO, or ENTDAA cannot store its complete result.
+Stimulus / Actions: Run `i3c_write_tx_fifo_underflow_vseq`, `i3c_read_rx_fifo_full_overflow_vseq`, and `i3c_entdaa_rx_fifo_partial_overflow_vseq`. Cover I3C and I2C, both I3C private-address modes, `toc=0/1`, TX FIFO empty/one-DWORD/late-refill cases, RX FIFO full/one-free-slot cases, partial-DWORD read lengths 1/2/3, a queued command after `toc=0`, and ENTDAA with 0/1/2 free entries for its 3-DWORD result. Run a successful transfer after each recovery policy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No garbage is transmitted or committed. Underflow/overflow forces STOP and suppresses continuation; at an I2C full-DWORD commit rejection the controller NACKs that byte before STOP. RESP is `Ovl` with matching TID, zero reserved bits, and actual length: bytes transmitted for TX underflow, bytes received through the rejected regular-read commit, or DAA-result bytes successfully committed (0/4/8). RX and ENTDAA paths recover after draining RX/RESP without SW reset. TX residual or late-refill data is cleared by waiting for idle and applying SW reset before the successful FIFO-backed recovery write.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `hci_queues`, `scl_generator`, `entdaa_controller`, RX FIFO, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_i3c_tx_underflow_resp_ovl`, `cp_i2c_tx_underflow_resp_ovl`, `cp_rx_commit_reject_latches_overflow`, `cp_rx_partial_dword_commit_overflow`, `cp_read_rx_overflow_blocks_data_and_continuation`, `cp_read_rx_overflow_requests_stop`, `cp_i2c_read_full_commit_boundary_nacks`, `cp_ovl_resp_matches_current_len`, `cp_i3c_read_rx_overflow_resp_ovl`, `cp_i2c_read_rx_overflow_resp_ovl`, `cp_entdaa_commit_reject_latches_overflow_and_stops`, `cp_entdaa_overflow_blocks_result_write`, `cp_entdaa_rx_overflow_resp_ovl`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_008</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify response write stalls safely.</t>
+    <t xml:space="preserve">Verify success and error response writes stall safely without loss, overwrite, or duplication.</t>
   </si>
   <si>
     <t xml:space="preserve">`resp_fifo_full_backpressure`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: RESP FIFO full before transaction completes.
-Stimulus / Actions: Complete a transfer while RESP full, then drain RESP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSM waits in response write phase; exactly one response is eventually written.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_resp_full`, `cp_stall_type`</t>
+    <t xml:space="preserve">Preconditions: RESP FIFO can be backdoor-filled before a response-producing command completes.
+Stimulus / Actions: Run `i3c_resp_fifo_full_backpressure_vseq`. First complete a successful regular write with `wroc=1` while RESP is full. Then repeat with a `wroc=0` immediate command that receives an address NACK. In each case, hold the FIFO full for multiple cycles, pop one prefilled entry, and drain the remaining entries plus the released response.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSM remains in `WriteResp`; response valid and descriptor data remain stable; FIFO pointers, depth, and all prefilled entries remain unchanged while blocked. One software pop releases exactly one pending response write. The prefilled entries retain FIFO order, the command response is appended once with the expected status/TID/length, and the final FIFO is empty. Successful `wroc=0` independence remains covered separately by ERR_012.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `hci_queues`, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_full_success_holds_pending_write`, `cp_resp_full_error_holds_pending_write`, `cp_resp_full_keeps_descriptor_stable`, `cp_resp_backpressure_release_writes_once`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_009</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify HC abort termination for I3C SDR, I2C regular, immediate, and ENTDAA transfers, including data integrity, response encoding, termination, and recovery policy.</t>
+    <t xml:space="preserve">Verify HC abort termination for I3C SDR, I2C regular, immediate, normal CCC, and ENTDAA transfers, including data integrity, response encoding, termination, priority, holdoff, and recovery policy.</t>
   </si>
   <si>
     <t xml:space="preserve">`resp_hc_abort_error`</t>
   </si>
   <si>
     <t xml:space="preserve">Preconditions: Controller can be aborted from selectable FSM states via persistent level bit `HC_CONTROL[29]` (ABORT).
-Stimulus / Actions: Run `i3c_write_abort_vseq`, `i3c_read_abort_vseq`, and `i2c_regular_abort_vseq` for early/deep/`toc=0` write and read transfers. Run `i3c_imm_abort_vseq` in I3C immediate mode with and without the broadcast-header preamble and in I2C immediate mode. Run `i3c_daa_hc_abort_vseq` during ENTDAA identity receive, assigned-address phase, and after one completed ENTDAA round. Also cover pre-bus, idle, priority, persistent-level, and CCC execution cases.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abort completes the defined byte boundary, forces STOP, suppresses continuation, preserves transmitted or committed data, and returns `HcAborted` with matching TID, zero reserved bits, and actual length. I3C/I2C regular writes can retain unfetched TX FIFO data and require clear-abort, idle, then SW reset for clean FIFO-backed recovery. I3C/I2C reads drain and verify committed RX data plus RESP; a following read succeeds without SW reset, which is needed only to discard residual state. Immediate data is descriptor-resident and similarly recovers without SW reset after clearing abort and draining RESP. ENTDAA abort drains any committed DAA result plus RESP, clears abort, and runs a following ENTDAA successfully without SW reset. I2C remains OD-only and uses controller NACK then STOP for read abort.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `csr_registers`, `hci_queues`, `scl_generator`, `bus_tx_flow`, `bus_rx_flow`, `entdaa_controller`, `entdaa_fsm`, RX FIFO, RESP FIFO, UVM scoreboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_hc_abort`, `cp_resp_err`, `cp_abort_entry_state`, `cp_resp_err_priority`, `cp_abort_stop_state`, `cp_private_start_prefix`, `cp_i2c_dir`, `cp_i2c_ack_seq`, `cp_daa_abort_point`, `cross_imm_x_device_type`</t>
+Stimulus / Actions: Run `i3c_write_abort_vseq`, `i3c_read_abort_vseq`, and `i2c_regular_abort_vseq` for early/deep/`toc=0` write and read transfers. Run `i3c_imm_abort_vseq` for private/broadcast-header I3C and I2C immediate transfers. Run `i3c_daa_hc_abort_vseq` during ENTDAA identity receive, assigned-address phase, and after one completed round, with a successful ENTDAA after every abort point. Run `i3c_hc_abort_policy_vseq` to hold abort at idle with a queued command, abort broadcast and direct ENEC at the completed-byte boundary, verify recovery without SW reset, and combine broadcast-header NACK with HC abort to verify `AddrHeader` priority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abort held at idle prevents CMD acceptance, START, and RESP generation until software clears it. Active abort completes the defined byte boundary, forces STOP, suppresses continuation, preserves transmitted or committed data, and returns `HcAborted` with matching TID, zero reserved bits, and actual length. A pre-existing higher-priority error overrides `HcAborted`. I3C/I2C regular writes can retain unfetched TX FIFO data and require clear-abort, idle, then SW reset for clean FIFO-backed recovery. I3C/I2C reads drain and verify committed RX data plus RESP and run a following read without SW reset. Immediate, normal CCC, and ENTDAA cases clear abort, drain committed data/RESP, and run a successful same-class command without SW reset. I2C remains OD-only and uses controller NACK then STOP for read abort.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `entdaa_fsm_sva`, `flow_active`, `csr_registers`, `hci_queues`, `scl_generator`, `bus_tx_flow`, `bus_rx_flow`, `entdaa_controller`, `entdaa_fsm`, RX FIFO, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_abort_entry_state`, `cp_abort_stop_state`, `cp_resp_err_priority`, `cp_abort_idle_blocks_command`, `cp_abort_error_priority_resp`, `cp_regular_write_abort_resp`, `cp_sdr_read_abort_resp`, `cp_i2c_read_abort_resp`, `cp_immediate_abort_resp`, `cp_ccc_abort_resp`, `cp_daa_abort_resp`, `cp_daa_abort_point`, `cp_private_start_prefix`, `cp_i2c_dir`, `cross_imm_x_device_type`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_010</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify pre-bus rejection of unsupported or invalid descriptor commands.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`invalid_descriptor_attr`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: CMD descriptors can be written directly; `cp=1` immediate CMD available for CCC opcode injection.
-Stimulus / Actions: (a) Issue `ComboTransfer`, reserved attr, HDR mode values, invalid mode encodings, and an `ImmediateDataTransfer` with `rnw=1`. (b) Issue representative unsupported CCC opcodes (`cp=1`, opcode outside ENEC/DISEC/ENTDAA) for both broadcast and direct forms (previously `ccc_unsupported_opcode_policy`).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**(b) Defined:** FSM rejects unsupported CCC opcode before any bus activity; RESP error is `NotSupported` (0xA); no CCC frame is emitted; queues drain cleanly. **(a) Clarification items:** no unbounded hang or illegal queue corruption; for `rnw=1` immediate the controller must not emit a read frame — it either ignores direction (forces write) or returns a specified error response; remaining subcases require sign-off once their expected behavior is specified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `i3c_pkg`, CMD descriptor parsing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_invalid_cmd`, `cp_imm`, `cp_unsupported_cmd`</t>
+    <t xml:space="preserve">Verify deterministic pre-DAT/pre-bus rejection, response encoding, and recovery for every unsupported descriptor class.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`i3c_invalid_descriptor_attr_vseq`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: CMD descriptors can be written directly; DAT[0] contains a valid I3C target for the recovery command.
+Stimulus / Actions: Sweep `ComboTransfer` and raw attrs `100..111`; Regular and Immediate with every mode other than `sdr0`; Immediate `rnw=1` and `dtt&gt;4`; Regular `cp=1`; unsupported broadcast CCC `02` and direct CCC `82`; and AddressAssignment with opcode other than ENTDAA. Include an invalid `wroc=0` descriptor and run a legal Immediate transfer after every rejection without SW reset.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each invalid command is rejected in `FetchDAT` without DAT read, START/RSTART/STOP, or bus TX/RX request. Exactly one RESP is written with `NotSupported` (0xA), matching TID, zero reserved bits, and length 0 regardless of WROC. CMD/RESP queues drain cleanly, TX/RX remain untouched, and every following legal command succeeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, CMD/RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_invalid_cmd`, `cp_imm`, `cp_unsupported_cmd`, `cp_invalid_cmd_rejected_before_access`, `cp_invalid_cmd_not_supported_resp`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_011</t>
@@ -1688,39 +1688,39 @@
     <t xml:space="preserve">`entdaa_invalid_descriptor_resp`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: CMD descriptors can be written directly; DAT entry exists but should not be used because the command is rejected before ENTDAA starts.
-Stimulus / Actions: Run `i3c_entdaa_invalid_descriptor_resp_vseq` with three subcases: `toc=0,wroc=1,dev_count=1`; `toc=1,wroc=0,dev_count=1`; and `toc=1,wroc=1,dev_count=0`.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No START, no `7'h7E+W` broadcast header, no ENTDAA opcode, and no DAA round are emitted. Exactly one RESP is written with status `NotSupported`, matching TID, reserved bits zero, and length 0. Queues drain cleanly and a following legal command can run.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, `i3c_pkg`, RESP FIFO, UVM scoreboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_addr_assign_desc`, `cp_resp_err`, `cp_tid`, `cp_resp_len`, `cp_no_bus_activity`</t>
+    <t xml:space="preserve">Preconditions: CMD descriptors can be written directly; DAT entries exist but must not be read because the command is rejected before ENTDAA starts.
+Stimulus / Actions: Run `i3c_entdaa_invalid_descriptor_resp_vseq` with four isolated subcases: `toc=0`; `wroc=0`; `dev_count=0`; and `dev_idx=31,dev_count=2` with `DatDepth=32`. Run a legal immediate transfer after every rejection without SW reset.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No DAT read, START/RSTART/STOP, bus TX/RX request, ENTDAA opcode, or DAA-controller activation occurs. Exactly one RESP is written with status `NotSupported`, matching TID, reserved bits zero, and length 0. Queues drain cleanly and every following legal command succeeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, `i3c_pkg`, CMD/RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_addr_assign_desc`, `cp_resp_err`, `cp_tid`, `cp_resp_len`, `cp_no_bus_activity`, `cp_addr_assign_invalid_rejected_before_access`, `cp_addr_assign_invalid_not_supported_resp`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_012</t>
   </si>
   <si>
-    <t xml:space="preserve">Document the `wroc` (response-on-completion) design gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`immediate_wroc_policy`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: CMD descriptors can be written directly.
-Stimulus / Actions: Issue immediate/regular commands with `wroc=0` and `wroc=1`.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">**Documented design gap — to be discussed / implemented later (not positive sign-off coverage).** RTL currently ignores the `wroc` field: `flow_active.sv` asserts `resp_queue_wvalid` unconditionally in `WriteResp` and `wroc` is never read, so a RESP descriptor is always written regardless of `wroc`. Behavior for `wroc=0` (suppress RESP write) is undefined until the project spec decides whether to implement it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`flow_active`, RESP FIFO, `csr_registers`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_wroc`</t>
+    <t xml:space="preserve">Verify response-on-completion suppression and error override for every supported command class.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`wroc_policy`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preconditions: DAT[0] is a responsive I3C target; CMD descriptors can set `wroc`; RESP FIFO can be backdoor-filled for the independence case.
+Stimulus / Actions: Run `i3c_wroc_policy_vseq`: issue successful regular, immediate, and immediate-CCC commands with `wroc=0/1`; run mixed-WROC commands; run a supported `toc=0,wroc=0` continuation while RESP is full; and NACK the address of a `wroc=0` immediate command.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Successful `wroc=1` commands write exactly one Success RESP. Successful `wroc=0` commands write no RESP and do not depend on RESP FIFO readiness. A supported `toc=0,wroc=0` command accepts its queued continuation without writing RESP, including while RESP is full; `wroc=1` continuation acceptance waits for RESP readiness. Address NACK and all other errors write a response regardless of WROC. Missing/unsupported continuation writes `NotSupported`. `AddressAssignment.wroc=0` remains invalid under ERR_011.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`flow_active_sva`, `flow_active`, RESP FIFO, UVM scoreboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_wroc0_success_suppresses_resp`, `cp_wroc1_success_enters_write_resp`, `cp_wroc0_error_override_writes_resp`, `cp_wroc0_continuation_ignores_resp_ready`, `cp_wroc1_continuation_waits_for_resp_ready`</t>
   </si>
   <si>
     <t xml:space="preserve">ERR_013</t>
@@ -2342,12 +2342,102 @@
     <t xml:space="preserve">0 bytes before abort, 1 word before abort, &gt;1 word before abort</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_abort_entry_state`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">idle/WaitForCmd holdoff; active preamble, CCC, transfer, and data states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_abort_stop_state`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preamble, normal CCC, and transfer data states that request STOP after HC abort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_err_priority`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`AddrHeader`, data NACK, DAA NACK, overflow, short read, and not-supported overriding `HcAborted`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_daa_abort_point`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identity receive, assigned-address phase, completed-round boundary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_abort_idle_blocks_command`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abort held in WaitForCmd with a command queued and no command pop/START</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_abort_error_priority_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HC abort coexists with a higher-priority error and the prioritized response is emitted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_regular_write_abort_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regular write emits exact `HcAborted` TID/reserved/actual-length fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_immediate_abort_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">immediate transfer emits exact `HcAborted` fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_ccc_abort_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broadcast/direct normal CCC emits exact `HcAborted` fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_daa_abort_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENTDAA emits exact `HcAborted` fields</t>
+  </si>
+  <si>
     <t xml:space="preserve">`cp_cmd_attr`</t>
   </si>
   <si>
     <t xml:space="preserve">`ImmediateDataTransfer`, `RegularTransfer`, `AddressAssignment`, `ComboTransfer/unsupported`, reserved</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_invalid_cmd`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invalid Regular, Immediate, AddressAssignment, Combo, and unsupported direct/internal attributes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_imm`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invalid Immediate combinations across `cp`, `rnw`, and mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_unsupported_cmd`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unsupported broadcast and direct immediate CCC opcode ranges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_invalid_cmd_rejected_before_access`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invalid descriptor reaches `FetchDAT` with all DAT and bus request outputs inactive, then enters `WriteResp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_invalid_cmd_not_supported_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invalid descriptor emits exact length-zero `NotSupported` response fields</t>
+  </si>
+  <si>
     <t xml:space="preserve">`cp_device_type`</t>
   </si>
   <si>
@@ -2396,10 +2486,40 @@
     <t xml:space="preserve">0 (regular transfers only — generates `Sr` on success or STOP on missing continuation), 1 (all transfer types — generates STOP; only valid option for immediate transfers)</t>
   </si>
   <si>
+    <t xml:space="preserve">`cp_wroc0_success_suppresses_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">successful regular, immediate, and immediate-CCC completion with no RESP write</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_wroc1_success_enters_write_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">successful response-producing completion enters `WriteResp` and asserts RESP valid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_wroc0_error_override_writes_resp`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error with `wroc=0` still enters `WriteResp` and asserts RESP valid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_wroc0_continuation_ignores_resp_ready`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supported `toc=0,wroc=0` continuation accepted while RESP is not ready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_wroc1_continuation_waits_for_resp_ready`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supported `toc=0,wroc=1` continuation held until RESP becomes ready</t>
+  </si>
+  <si>
     <t xml:space="preserve">`cp_resp_err`</t>
   </si>
   <si>
-    <t xml:space="preserve">Success, AddrHeader, Nack, Ovl, I3cShortReadErr, unreachable-defined-codes</t>
+    <t xml:space="preserve">Success, AddrHeader, Nack, Ovl, I3cShortReadErr, I2cDataNackOrI3cBusAborted, unreachable-defined-codes</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_addr_ack`</t>
@@ -2508,6 +2628,30 @@
   </si>
   <si>
     <t xml:space="preserve">TX empty, RX full, RESP full, none</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_full_success_holds_pending_write`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A successful `wroc=1` response remains valid in `WriteResp` while RESP is full.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_full_error_holds_pending_write`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An error response remains valid in `WriteResp` while RESP is full, including when the command has `wroc=0`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_full_keeps_descriptor_stable`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response status, TID, reserved bits, and length remain stable across a blocked cycle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`cp_resp_backpressure_release_writes_once`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A previously blocked response handshakes when space appears and exits `WriteResp` on the following cycle.</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_ccc_opcode`</t>
@@ -4855,25 +4999,25 @@
         <v>465</v>
       </c>
       <c r="D68" t="s" s="2">
-        <v>466</v>
+        <v>416</v>
       </c>
       <c r="E68" t="s" s="2">
         <v>465</v>
       </c>
       <c r="F68" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="G68" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="G68" t="s" s="2">
+      <c r="H68" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I68" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="H68" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I68" t="s" s="2">
+      <c r="J68" t="s" s="2">
         <v>469</v>
-      </c>
-      <c r="J68" t="s" s="2">
-        <v>470</v>
       </c>
     </row>
     <row r="69">
@@ -4881,31 +5025,31 @@
         <v>19</v>
       </c>
       <c r="B69" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="C69" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="C69" t="s" s="2">
+      <c r="D69" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="D69" t="s" s="2">
+      <c r="E69" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="F69" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="E69" t="s" s="2">
-        <v>472</v>
-      </c>
-      <c r="F69" t="s" s="2">
+      <c r="G69" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="G69" t="s" s="2">
+      <c r="H69" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I69" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="J69" t="s" s="2">
         <v>475</v>
-      </c>
-      <c r="H69" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I69" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="J69" t="s" s="2">
-        <v>476</v>
       </c>
     </row>
     <row r="70">
@@ -4913,31 +5057,31 @@
         <v>19</v>
       </c>
       <c r="B70" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="C70" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="C70" t="s" s="2">
+      <c r="D70" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="D70" t="s" s="2">
+      <c r="E70" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="F70" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="E70" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="F70" t="s" s="2">
+      <c r="G70" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="G70" t="s" s="2">
+      <c r="H70" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I70" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="J70" t="s" s="2">
         <v>481</v>
-      </c>
-      <c r="H70" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I70" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="J70" t="s" s="2">
-        <v>482</v>
       </c>
     </row>
     <row r="71">
@@ -4945,31 +5089,31 @@
         <v>19</v>
       </c>
       <c r="B71" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="C71" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="C71" t="s" s="2">
+      <c r="D71" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="D71" t="s" s="2">
+      <c r="E71" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="F71" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="E71" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="F71" t="s" s="2">
+      <c r="G71" t="s" s="2">
         <v>486</v>
       </c>
-      <c r="G71" t="s" s="2">
+      <c r="H71" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I71" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="H71" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I71" t="s" s="2">
+      <c r="J71" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="J71" t="s" s="2">
-        <v>489</v>
       </c>
     </row>
     <row r="72">
@@ -4977,31 +5121,31 @@
         <v>19</v>
       </c>
       <c r="B72" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="C72" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="C72" t="s" s="2">
+      <c r="D72" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="D72" t="s" s="2">
+      <c r="E72" t="s" s="2">
+        <v>490</v>
+      </c>
+      <c r="F72" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="E72" t="s" s="2">
-        <v>491</v>
-      </c>
-      <c r="F72" t="s" s="2">
+      <c r="G72" t="s" s="2">
         <v>493</v>
       </c>
-      <c r="G72" t="s" s="2">
+      <c r="H72" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I72" t="s" s="2">
         <v>494</v>
       </c>
-      <c r="H72" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I72" t="s" s="2">
+      <c r="J72" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="J72" t="s" s="2">
-        <v>496</v>
       </c>
     </row>
     <row r="73">
@@ -5009,31 +5153,31 @@
         <v>19</v>
       </c>
       <c r="B73" t="s" s="2">
+        <v>496</v>
+      </c>
+      <c r="C73" t="s" s="2">
         <v>497</v>
       </c>
-      <c r="C73" t="s" s="2">
+      <c r="D73" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="E73" t="s" s="2">
+        <v>497</v>
+      </c>
+      <c r="F73" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="D73" t="s" s="2">
+      <c r="G73" t="s" s="2">
         <v>499</v>
       </c>
-      <c r="E73" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="F73" t="s" s="2">
+      <c r="H73" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I73" t="s" s="2">
         <v>500</v>
       </c>
-      <c r="G73" t="s" s="2">
+      <c r="J73" t="s" s="2">
         <v>501</v>
-      </c>
-      <c r="H73" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I73" t="s" s="2">
-        <v>495</v>
-      </c>
-      <c r="J73" t="s" s="2">
-        <v>502</v>
       </c>
     </row>
     <row r="74">
@@ -5041,31 +5185,31 @@
         <v>19</v>
       </c>
       <c r="B74" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="C74" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="C74" t="s" s="2">
+      <c r="D74" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="D74" t="s" s="2">
+      <c r="E74" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="F74" t="s" s="2">
         <v>505</v>
       </c>
-      <c r="E74" t="s" s="2">
-        <v>504</v>
-      </c>
-      <c r="F74" t="s" s="2">
+      <c r="G74" t="s" s="2">
         <v>506</v>
       </c>
-      <c r="G74" t="s" s="2">
+      <c r="H74" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I74" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="H74" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I74" t="s" s="2">
+      <c r="J74" t="s" s="2">
         <v>508</v>
-      </c>
-      <c r="J74" t="s" s="2">
-        <v>509</v>
       </c>
     </row>
     <row r="75">
@@ -5073,28 +5217,28 @@
         <v>19</v>
       </c>
       <c r="B75" t="s" s="2">
+        <v>509</v>
+      </c>
+      <c r="C75" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="C75" t="s" s="2">
+      <c r="D75" t="s" s="2">
         <v>511</v>
       </c>
-      <c r="D75" t="s" s="2">
+      <c r="E75" t="s" s="2">
+        <v>510</v>
+      </c>
+      <c r="F75" t="s" s="2">
         <v>512</v>
       </c>
-      <c r="E75" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="F75" t="s" s="2">
+      <c r="G75" t="s" s="2">
         <v>513</v>
       </c>
-      <c r="G75" t="s" s="2">
+      <c r="H75" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I75" t="s" s="2">
         <v>514</v>
-      </c>
-      <c r="H75" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I75" t="s" s="2">
-        <v>455</v>
       </c>
       <c r="J75" t="s" s="2">
         <v>515</v>
@@ -5155,7 +5299,7 @@
         <v>527</v>
       </c>
       <c r="H77" t="s" s="2">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="I77" t="s" s="2">
         <v>528</v>
@@ -5219,7 +5363,7 @@
         <v>541</v>
       </c>
       <c r="H79" t="s" s="2">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="I79" t="s" s="2">
         <v>542</v>
@@ -6477,10 +6621,10 @@
         <v>19</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>233</v>
+        <v>793</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>793</v>
+        <v>794</v>
       </c>
     </row>
     <row r="33">
@@ -6488,10 +6632,10 @@
         <v>19</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>462</v>
+        <v>795</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>794</v>
+        <v>796</v>
       </c>
     </row>
     <row r="34">
@@ -6499,10 +6643,10 @@
         <v>19</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>796</v>
+        <v>798</v>
       </c>
     </row>
     <row r="35">
@@ -6510,10 +6654,10 @@
         <v>19</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>798</v>
+        <v>800</v>
       </c>
     </row>
     <row r="36">
@@ -6521,10 +6665,10 @@
         <v>19</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>800</v>
+        <v>802</v>
       </c>
     </row>
     <row r="37">
@@ -6532,10 +6676,10 @@
         <v>19</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>802</v>
+        <v>804</v>
       </c>
     </row>
     <row r="38">
@@ -6543,10 +6687,10 @@
         <v>19</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>804</v>
+        <v>806</v>
       </c>
     </row>
     <row r="39">
@@ -6554,10 +6698,10 @@
         <v>19</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>806</v>
+        <v>808</v>
       </c>
     </row>
     <row r="40">
@@ -6565,10 +6709,10 @@
         <v>19</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>550</v>
+        <v>809</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>807</v>
+        <v>810</v>
       </c>
     </row>
     <row r="41">
@@ -6576,21 +6720,21 @@
         <v>19</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>19</v>
+        <v>811</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>19</v>
+        <v>812</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>808</v>
+        <v>19</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>19</v>
+        <v>813</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>19</v>
+        <v>814</v>
       </c>
     </row>
     <row r="43">
@@ -6598,10 +6742,10 @@
         <v>19</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="C43" t="s" s="2">
-        <v>810</v>
+        <v>816</v>
       </c>
     </row>
     <row r="44">
@@ -6609,10 +6753,10 @@
         <v>19</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>812</v>
+        <v>818</v>
       </c>
     </row>
     <row r="45">
@@ -6620,10 +6764,10 @@
         <v>19</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>813</v>
+        <v>819</v>
       </c>
       <c r="C45" t="s" s="2">
-        <v>814</v>
+        <v>820</v>
       </c>
     </row>
     <row r="46">
@@ -6631,10 +6775,10 @@
         <v>19</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="C46" t="s" s="2">
-        <v>816</v>
+        <v>822</v>
       </c>
     </row>
     <row r="47">
@@ -6642,10 +6786,10 @@
         <v>19</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>818</v>
+        <v>824</v>
       </c>
     </row>
     <row r="48">
@@ -6653,10 +6797,10 @@
         <v>19</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>819</v>
+        <v>825</v>
       </c>
       <c r="C48" t="s" s="2">
-        <v>820</v>
+        <v>826</v>
       </c>
     </row>
     <row r="49">
@@ -6664,10 +6808,10 @@
         <v>19</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="50">
@@ -6675,10 +6819,10 @@
         <v>19</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>824</v>
+        <v>830</v>
       </c>
     </row>
     <row r="51">
@@ -6686,10 +6830,10 @@
         <v>19</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="C51" t="s" s="2">
-        <v>826</v>
+        <v>832</v>
       </c>
     </row>
     <row r="52">
@@ -6697,10 +6841,10 @@
         <v>19</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>827</v>
+        <v>233</v>
       </c>
       <c r="C52" t="s" s="2">
-        <v>828</v>
+        <v>833</v>
       </c>
     </row>
     <row r="53">
@@ -6708,10 +6852,10 @@
         <v>19</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>829</v>
+        <v>462</v>
       </c>
       <c r="C53" t="s" s="2">
-        <v>830</v>
+        <v>834</v>
       </c>
     </row>
     <row r="54">
@@ -6719,10 +6863,10 @@
         <v>19</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="C54" t="s" s="2">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="55">
@@ -6730,10 +6874,10 @@
         <v>19</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C55" t="s" s="2">
-        <v>834</v>
+        <v>838</v>
       </c>
     </row>
     <row r="56">
@@ -6741,10 +6885,274 @@
         <v>19</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="C56" t="s" s="2">
-        <v>836</v>
+        <v>840</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>841</v>
+      </c>
+      <c r="C57" t="s" s="2">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>843</v>
+      </c>
+      <c r="C58" t="s" s="2">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>845</v>
+      </c>
+      <c r="C59" t="s" s="2">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>847</v>
+      </c>
+      <c r="C60" t="s" s="2">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>849</v>
+      </c>
+      <c r="C61" t="s" s="2">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>851</v>
+      </c>
+      <c r="C62" t="s" s="2">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B63" t="s" s="2">
+        <v>853</v>
+      </c>
+      <c r="C63" t="s" s="2">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B64" t="s" s="2">
+        <v>550</v>
+      </c>
+      <c r="C64" t="s" s="2">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="C65" t="s" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="2">
+        <v>856</v>
+      </c>
+      <c r="B66" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="C66" t="s" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B67" t="s" s="2">
+        <v>857</v>
+      </c>
+      <c r="C67" t="s" s="2">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B68" t="s" s="2">
+        <v>859</v>
+      </c>
+      <c r="C68" t="s" s="2">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B69" t="s" s="2">
+        <v>861</v>
+      </c>
+      <c r="C69" t="s" s="2">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B70" t="s" s="2">
+        <v>863</v>
+      </c>
+      <c r="C70" t="s" s="2">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B71" t="s" s="2">
+        <v>865</v>
+      </c>
+      <c r="C71" t="s" s="2">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B72" t="s" s="2">
+        <v>867</v>
+      </c>
+      <c r="C72" t="s" s="2">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B73" t="s" s="2">
+        <v>869</v>
+      </c>
+      <c r="C73" t="s" s="2">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B74" t="s" s="2">
+        <v>871</v>
+      </c>
+      <c r="C74" t="s" s="2">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B75" t="s" s="2">
+        <v>873</v>
+      </c>
+      <c r="C75" t="s" s="2">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B76" t="s" s="2">
+        <v>875</v>
+      </c>
+      <c r="C76" t="s" s="2">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B77" t="s" s="2">
+        <v>877</v>
+      </c>
+      <c r="C77" t="s" s="2">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B78" t="s" s="2">
+        <v>879</v>
+      </c>
+      <c r="C78" t="s" s="2">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>881</v>
+      </c>
+      <c r="C79" t="s" s="2">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B80" t="s" s="2">
+        <v>883</v>
+      </c>
+      <c r="C80" t="s" s="2">
+        <v>884</v>
       </c>
     </row>
   </sheetData>
@@ -6759,15 +7167,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>837</v>
+        <v>885</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>838</v>
+        <v>886</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>839</v>
+        <v>887</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>690</v>
@@ -6778,7 +7186,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>840</v>
+        <v>888</v>
       </c>
       <c r="B3" t="s" s="2">
         <v>697</v>
@@ -6789,7 +7197,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>841</v>
+        <v>889</v>
       </c>
       <c r="B4" t="s" s="2">
         <v>702</v>
@@ -6819,7 +7227,7 @@
         <v>4</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>842</v>
+        <v>890</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Add functional coverage model
</commit_message>
<xml_diff>
--- a/docs/test_plan/I3C_Testplan.xlsx
+++ b/docs/test_plan/I3C_Testplan.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="883">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -1767,17 +1767,17 @@
     <t xml:space="preserve">ERR_015</t>
   </si>
   <si>
-    <t xml:space="preserve">Clarify SW reset during active transfer.</t>
+    <t xml:space="preserve">Verify deterministic SW reset behavior during active transfer.</t>
   </si>
   <si>
     <t xml:space="preserve">`sw_reset_while_busy_policy`</t>
   </si>
   <si>
-    <t xml:space="preserve">Preconditions: Transfer in progress.
-Stimulus / Actions: Assert `RESET_CONTROL[0]` (SOFT_RST) while not idle.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If the spec leaves this undefined, the test records a spec gap and recommends SW only reset when `FSM_IDLE=1`; it is not positive sign-off coverage until a busy-reset policy is specified.</t>
+    <t xml:space="preserve">Preconditions: Transfer in progress with queued continuation work.
+Stimulus / Actions: Assert `RESET_CONTROL[0]` (SOFT_RST) while `HC_STATUS[FSM_IDLE]=0`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Busy SOFT_RST is accepted as a no-op: no `sw_reset` pulse, no queue flush, no CSR staging clear, no protocol FSM reset, and the active plus queued transfers complete normally. Idle SOFT_RST behavior remains covered by CSR_008/CSR_009.</t>
   </si>
   <si>
     <t xml:space="preserve">`csr_registers`, `hci_queues`, `flow_active`</t>
@@ -1814,32 +1814,10 @@
     <t xml:space="preserve">ARB_001</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify ENTDAA bit-level receiver samples wired bus.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`entdaa_single_bit_arbitration_observe`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions: DAA target drives known PID bits.
-Stimulus / Actions: During ENTDAA, observe each PID/BCR/DCR bit sampled by `bus_rx_flow`.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Captured 64-bit identity matches bus data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`entdaa_fsm`, `bus_rx_flow`, bus model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`cp_daa_bit_pos`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARB_002</t>
-  </si>
-  <si>
     <t xml:space="preserve">Verify true multi-target ENTDAA arbitration.</t>
   </si>
   <si>
-    <t xml:space="preserve">`entdaa_multi_target_arbitration_future`</t>
+    <t xml:space="preserve">`i3c_entdaa_multi_target_arbitration_vseq`</t>
   </si>
   <si>
     <t xml:space="preserve">Preconditions: UVM bus model supports simultaneous target driving.
@@ -1849,16 +1827,13 @@
     <t xml:space="preserve">Master assigns the arbitration winner first; losing targets are not assigned in that round and retry in later rounds. The two-target case is the minimum subcase of this multi-target coverage item, not a separate testcase.</t>
   </si>
   <si>
-    <t xml:space="preserve">Future</t>
-  </si>
-  <si>
     <t xml:space="preserve">UVM I3C agent, bus, `entdaa_fsm`</t>
   </si>
   <si>
     <t xml:space="preserve">`cp_daa_arbitration`</t>
   </si>
   <si>
-    <t xml:space="preserve">ARB_003</t>
+    <t xml:space="preserve">ARB_002</t>
   </si>
   <si>
     <t xml:space="preserve">Verify STOP detection during active command.</t>
@@ -1880,7 +1855,7 @@
     <t xml:space="preserve">`cp_unexpected_bus_event`</t>
   </si>
   <si>
-    <t xml:space="preserve">ARB_004</t>
+    <t xml:space="preserve">ARB_003</t>
   </si>
   <si>
     <t xml:space="preserve">Verify controller behavior if command starts on busy bus.</t>
@@ -5555,13 +5530,13 @@
         <v>583</v>
       </c>
       <c r="H85" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I85" t="s" s="2">
         <v>584</v>
       </c>
-      <c r="I85" t="s" s="2">
+      <c r="J85" t="s" s="2">
         <v>585</v>
-      </c>
-      <c r="J85" t="s" s="2">
-        <v>586</v>
       </c>
     </row>
     <row r="86">
@@ -5569,60 +5544,60 @@
         <v>19</v>
       </c>
       <c r="B86" t="s" s="2">
+        <v>586</v>
+      </c>
+      <c r="C86" t="s" s="2">
         <v>587</v>
       </c>
-      <c r="C86" t="s" s="2">
+      <c r="D86" t="s" s="2">
         <v>588</v>
       </c>
-      <c r="D86" t="s" s="2">
+      <c r="E86" t="s" s="2">
+        <v>587</v>
+      </c>
+      <c r="F86" t="s" s="2">
         <v>589</v>
       </c>
-      <c r="E86" t="s" s="2">
-        <v>588</v>
-      </c>
-      <c r="F86" t="s" s="2">
+      <c r="G86" t="s" s="2">
         <v>590</v>
-      </c>
-      <c r="G86" t="s" s="2">
-        <v>591</v>
       </c>
       <c r="H86" t="s" s="2">
         <v>59</v>
       </c>
       <c r="I86" t="s" s="2">
-        <v>592</v>
+        <v>569</v>
       </c>
       <c r="J86" t="s" s="2">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>19</v>
+        <v>592</v>
       </c>
       <c r="B87" t="s" s="2">
+        <v>593</v>
+      </c>
+      <c r="C87" t="s" s="2">
         <v>594</v>
       </c>
-      <c r="C87" t="s" s="2">
+      <c r="D87" t="s" s="2">
         <v>595</v>
       </c>
-      <c r="D87" t="s" s="2">
+      <c r="E87" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="F87" t="s" s="2">
         <v>596</v>
       </c>
-      <c r="E87" t="s" s="2">
-        <v>595</v>
-      </c>
-      <c r="F87" t="s" s="2">
+      <c r="G87" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="G87" t="s" s="2">
+      <c r="H87" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I87" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="H87" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="I87" t="s" s="2">
-        <v>569</v>
       </c>
       <c r="J87" t="s" s="2">
         <v>599</v>
@@ -5630,34 +5605,34 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B88" t="s" s="2">
         <v>600</v>
       </c>
-      <c r="B88" t="s" s="2">
+      <c r="C88" t="s" s="2">
         <v>601</v>
       </c>
-      <c r="C88" t="s" s="2">
+      <c r="D88" t="s" s="2">
         <v>602</v>
       </c>
-      <c r="D88" t="s" s="2">
+      <c r="E88" t="s" s="2">
+        <v>601</v>
+      </c>
+      <c r="F88" t="s" s="2">
         <v>603</v>
       </c>
-      <c r="E88" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="F88" t="s" s="2">
+      <c r="G88" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="G88" t="s" s="2">
+      <c r="H88" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I88" t="s" s="2">
         <v>605</v>
       </c>
-      <c r="H88" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I88" t="s" s="2">
+      <c r="J88" t="s" s="2">
         <v>606</v>
-      </c>
-      <c r="J88" t="s" s="2">
-        <v>607</v>
       </c>
     </row>
     <row r="89">
@@ -5665,31 +5640,31 @@
         <v>19</v>
       </c>
       <c r="B89" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="C89" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="C89" t="s" s="2">
+      <c r="D89" t="s" s="2">
         <v>609</v>
       </c>
-      <c r="D89" t="s" s="2">
+      <c r="E89" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="F89" t="s" s="2">
         <v>610</v>
       </c>
-      <c r="E89" t="s" s="2">
-        <v>609</v>
-      </c>
-      <c r="F89" t="s" s="2">
+      <c r="G89" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="G89" t="s" s="2">
+      <c r="H89" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I89" t="s" s="2">
         <v>612</v>
       </c>
-      <c r="H89" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I89" t="s" s="2">
-        <v>613</v>
-      </c>
       <c r="J89" t="s" s="2">
-        <v>614</v>
+        <v>606</v>
       </c>
     </row>
     <row r="90">
@@ -5697,31 +5672,31 @@
         <v>19</v>
       </c>
       <c r="B90" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="C90" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="D90" t="s" s="2">
         <v>615</v>
       </c>
-      <c r="C90" t="s" s="2">
+      <c r="E90" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="F90" t="s" s="2">
         <v>616</v>
       </c>
-      <c r="D90" t="s" s="2">
+      <c r="G90" t="s" s="2">
         <v>617</v>
       </c>
-      <c r="E90" t="s" s="2">
-        <v>616</v>
-      </c>
-      <c r="F90" t="s" s="2">
+      <c r="H90" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I90" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="G90" t="s" s="2">
+      <c r="J90" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="H90" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I90" t="s" s="2">
-        <v>620</v>
-      </c>
-      <c r="J90" t="s" s="2">
-        <v>614</v>
       </c>
     </row>
     <row r="91">
@@ -5729,31 +5704,31 @@
         <v>19</v>
       </c>
       <c r="B91" t="s" s="2">
+        <v>620</v>
+      </c>
+      <c r="C91" t="s" s="2">
         <v>621</v>
       </c>
-      <c r="C91" t="s" s="2">
+      <c r="D91" t="s" s="2">
         <v>622</v>
       </c>
-      <c r="D91" t="s" s="2">
+      <c r="E91" t="s" s="2">
+        <v>621</v>
+      </c>
+      <c r="F91" t="s" s="2">
         <v>623</v>
       </c>
-      <c r="E91" t="s" s="2">
-        <v>622</v>
-      </c>
-      <c r="F91" t="s" s="2">
+      <c r="G91" t="s" s="2">
         <v>624</v>
       </c>
-      <c r="G91" t="s" s="2">
+      <c r="H91" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I91" t="s" s="2">
+        <v>618</v>
+      </c>
+      <c r="J91" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="H91" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I91" t="s" s="2">
-        <v>626</v>
-      </c>
-      <c r="J91" t="s" s="2">
-        <v>627</v>
       </c>
     </row>
     <row r="92">
@@ -5761,31 +5736,31 @@
         <v>19</v>
       </c>
       <c r="B92" t="s" s="2">
+        <v>626</v>
+      </c>
+      <c r="C92" t="s" s="2">
+        <v>627</v>
+      </c>
+      <c r="D92" t="s" s="2">
         <v>628</v>
       </c>
-      <c r="C92" t="s" s="2">
+      <c r="E92" t="s" s="2">
+        <v>627</v>
+      </c>
+      <c r="F92" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="D92" t="s" s="2">
+      <c r="G92" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="E92" t="s" s="2">
-        <v>629</v>
-      </c>
-      <c r="F92" t="s" s="2">
+      <c r="H92" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I92" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="G92" t="s" s="2">
+      <c r="J92" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="H92" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="I92" t="s" s="2">
-        <v>626</v>
-      </c>
-      <c r="J92" t="s" s="2">
-        <v>633</v>
       </c>
     </row>
     <row r="93">
@@ -5793,31 +5768,31 @@
         <v>19</v>
       </c>
       <c r="B93" t="s" s="2">
+        <v>633</v>
+      </c>
+      <c r="C93" t="s" s="2">
         <v>634</v>
       </c>
-      <c r="C93" t="s" s="2">
+      <c r="D93" t="s" s="2">
         <v>635</v>
       </c>
-      <c r="D93" t="s" s="2">
+      <c r="E93" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="F93" t="s" s="2">
         <v>636</v>
       </c>
-      <c r="E93" t="s" s="2">
-        <v>635</v>
-      </c>
-      <c r="F93" t="s" s="2">
+      <c r="G93" t="s" s="2">
         <v>637</v>
       </c>
-      <c r="G93" t="s" s="2">
+      <c r="H93" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I93" t="s" s="2">
         <v>638</v>
       </c>
-      <c r="H93" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I93" t="s" s="2">
+      <c r="J93" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="J93" t="s" s="2">
-        <v>640</v>
       </c>
     </row>
     <row r="94">
@@ -5825,36 +5800,36 @@
         <v>19</v>
       </c>
       <c r="B94" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="C94" t="s" s="2">
         <v>641</v>
       </c>
-      <c r="C94" t="s" s="2">
+      <c r="D94" t="s" s="2">
         <v>642</v>
       </c>
-      <c r="D94" t="s" s="2">
+      <c r="E94" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="F94" t="s" s="2">
         <v>643</v>
       </c>
-      <c r="E94" t="s" s="2">
-        <v>642</v>
-      </c>
-      <c r="F94" t="s" s="2">
+      <c r="G94" t="s" s="2">
         <v>644</v>
       </c>
-      <c r="G94" t="s" s="2">
+      <c r="H94" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I94" t="s" s="2">
         <v>645</v>
       </c>
-      <c r="H94" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I94" t="s" s="2">
+      <c r="J94" t="s" s="2">
         <v>646</v>
-      </c>
-      <c r="J94" t="s" s="2">
-        <v>647</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>19</v>
+        <v>647</v>
       </c>
       <c r="B95" t="s" s="2">
         <v>648</v>
@@ -5875,7 +5850,7 @@
         <v>652</v>
       </c>
       <c r="H95" t="s" s="2">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="I95" t="s" s="2">
         <v>653</v>
@@ -5886,34 +5861,34 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B96" t="s" s="2">
         <v>655</v>
       </c>
-      <c r="B96" t="s" s="2">
+      <c r="C96" t="s" s="2">
         <v>656</v>
       </c>
-      <c r="C96" t="s" s="2">
+      <c r="D96" t="s" s="2">
         <v>657</v>
       </c>
-      <c r="D96" t="s" s="2">
+      <c r="E96" t="s" s="2">
+        <v>656</v>
+      </c>
+      <c r="F96" t="s" s="2">
         <v>658</v>
       </c>
-      <c r="E96" t="s" s="2">
-        <v>657</v>
-      </c>
-      <c r="F96" t="s" s="2">
+      <c r="G96" t="s" s="2">
         <v>659</v>
       </c>
-      <c r="G96" t="s" s="2">
+      <c r="H96" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I96" t="s" s="2">
         <v>660</v>
       </c>
-      <c r="H96" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I96" t="s" s="2">
+      <c r="J96" t="s" s="2">
         <v>661</v>
-      </c>
-      <c r="J96" t="s" s="2">
-        <v>662</v>
       </c>
     </row>
     <row r="97">
@@ -5921,31 +5896,31 @@
         <v>19</v>
       </c>
       <c r="B97" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="C97" t="s" s="2">
         <v>663</v>
       </c>
-      <c r="C97" t="s" s="2">
+      <c r="D97" t="s" s="2">
         <v>664</v>
       </c>
-      <c r="D97" t="s" s="2">
+      <c r="E97" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="F97" t="s" s="2">
         <v>665</v>
       </c>
-      <c r="E97" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="F97" t="s" s="2">
+      <c r="G97" t="s" s="2">
         <v>666</v>
       </c>
-      <c r="G97" t="s" s="2">
+      <c r="H97" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I97" t="s" s="2">
+        <v>653</v>
+      </c>
+      <c r="J97" t="s" s="2">
         <v>667</v>
-      </c>
-      <c r="H97" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I97" t="s" s="2">
-        <v>668</v>
-      </c>
-      <c r="J97" t="s" s="2">
-        <v>669</v>
       </c>
     </row>
     <row r="98">
@@ -5953,31 +5928,31 @@
         <v>19</v>
       </c>
       <c r="B98" t="s" s="2">
+        <v>668</v>
+      </c>
+      <c r="C98" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="D98" t="s" s="2">
         <v>670</v>
       </c>
-      <c r="C98" t="s" s="2">
+      <c r="E98" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="F98" t="s" s="2">
         <v>671</v>
       </c>
-      <c r="D98" t="s" s="2">
+      <c r="G98" t="s" s="2">
         <v>672</v>
       </c>
-      <c r="E98" t="s" s="2">
-        <v>671</v>
-      </c>
-      <c r="F98" t="s" s="2">
+      <c r="H98" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I98" t="s" s="2">
         <v>673</v>
       </c>
-      <c r="G98" t="s" s="2">
+      <c r="J98" t="s" s="2">
         <v>674</v>
-      </c>
-      <c r="H98" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I98" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="J98" t="s" s="2">
-        <v>675</v>
       </c>
     </row>
     <row r="99">
@@ -5985,31 +5960,31 @@
         <v>19</v>
       </c>
       <c r="B99" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="C99" t="s" s="2">
         <v>676</v>
       </c>
-      <c r="C99" t="s" s="2">
+      <c r="D99" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="D99" t="s" s="2">
+      <c r="E99" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="F99" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="E99" t="s" s="2">
-        <v>677</v>
-      </c>
-      <c r="F99" t="s" s="2">
+      <c r="G99" t="s" s="2">
         <v>679</v>
       </c>
-      <c r="G99" t="s" s="2">
+      <c r="H99" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="I99" t="s" s="2">
+        <v>653</v>
+      </c>
+      <c r="J99" t="s" s="2">
         <v>680</v>
-      </c>
-      <c r="H99" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I99" t="s" s="2">
-        <v>681</v>
-      </c>
-      <c r="J99" t="s" s="2">
-        <v>682</v>
       </c>
     </row>
     <row r="100">
@@ -6017,31 +5992,31 @@
         <v>19</v>
       </c>
       <c r="B100" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="C100" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="D100" t="s" s="2">
         <v>683</v>
       </c>
-      <c r="C100" t="s" s="2">
+      <c r="E100" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="F100" t="s" s="2">
         <v>684</v>
       </c>
-      <c r="D100" t="s" s="2">
+      <c r="G100" t="s" s="2">
         <v>685</v>
       </c>
-      <c r="E100" t="s" s="2">
-        <v>684</v>
-      </c>
-      <c r="F100" t="s" s="2">
+      <c r="H100" t="s" s="2">
         <v>686</v>
       </c>
-      <c r="G100" t="s" s="2">
+      <c r="I100" t="s" s="2">
+        <v>653</v>
+      </c>
+      <c r="J100" t="s" s="2">
         <v>687</v>
-      </c>
-      <c r="H100" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="I100" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="J100" t="s" s="2">
-        <v>688</v>
       </c>
     </row>
     <row r="101">
@@ -6049,31 +6024,31 @@
         <v>19</v>
       </c>
       <c r="B101" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="C101" t="s" s="2">
         <v>689</v>
       </c>
-      <c r="C101" t="s" s="2">
+      <c r="D101" t="s" s="2">
         <v>690</v>
       </c>
-      <c r="D101" t="s" s="2">
+      <c r="E101" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="F101" t="s" s="2">
         <v>691</v>
       </c>
-      <c r="E101" t="s" s="2">
-        <v>690</v>
-      </c>
-      <c r="F101" t="s" s="2">
+      <c r="G101" t="s" s="2">
         <v>692</v>
       </c>
-      <c r="G101" t="s" s="2">
-        <v>693</v>
-      </c>
       <c r="H101" t="s" s="2">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="I101" t="s" s="2">
-        <v>661</v>
+        <v>653</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>695</v>
+        <v>687</v>
       </c>
     </row>
     <row r="102">
@@ -6081,60 +6056,60 @@
         <v>19</v>
       </c>
       <c r="B102" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="C102" t="s" s="2">
+        <v>694</v>
+      </c>
+      <c r="D102" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="E102" t="s" s="2">
+        <v>694</v>
+      </c>
+      <c r="F102" t="s" s="2">
         <v>696</v>
       </c>
-      <c r="C102" t="s" s="2">
+      <c r="G102" t="s" s="2">
         <v>697</v>
       </c>
-      <c r="D102" t="s" s="2">
+      <c r="H102" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="I102" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="J102" t="s" s="2">
         <v>698</v>
-      </c>
-      <c r="E102" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="F102" t="s" s="2">
-        <v>699</v>
-      </c>
-      <c r="G102" t="s" s="2">
-        <v>700</v>
-      </c>
-      <c r="H102" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="I102" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="J102" t="s" s="2">
-        <v>695</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>19</v>
+        <v>699</v>
       </c>
       <c r="B103" t="s" s="2">
+        <v>700</v>
+      </c>
+      <c r="C103" t="s" s="2">
         <v>701</v>
       </c>
-      <c r="C103" t="s" s="2">
+      <c r="D103" t="s" s="2">
         <v>702</v>
       </c>
-      <c r="D103" t="s" s="2">
+      <c r="E103" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="F103" t="s" s="2">
         <v>703</v>
       </c>
-      <c r="E103" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="F103" t="s" s="2">
+      <c r="G103" t="s" s="2">
         <v>704</v>
       </c>
-      <c r="G103" t="s" s="2">
+      <c r="H103" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="I103" t="s" s="2">
         <v>705</v>
-      </c>
-      <c r="H103" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="I103" t="s" s="2">
-        <v>342</v>
       </c>
       <c r="J103" t="s" s="2">
         <v>706</v>
@@ -6142,34 +6117,34 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B104" t="s" s="2">
         <v>707</v>
       </c>
-      <c r="B104" t="s" s="2">
+      <c r="C104" t="s" s="2">
         <v>708</v>
       </c>
-      <c r="C104" t="s" s="2">
+      <c r="D104" t="s" s="2">
         <v>709</v>
       </c>
-      <c r="D104" t="s" s="2">
+      <c r="E104" t="s" s="2">
+        <v>708</v>
+      </c>
+      <c r="F104" t="s" s="2">
         <v>710</v>
       </c>
-      <c r="E104" t="s" s="2">
-        <v>709</v>
-      </c>
-      <c r="F104" t="s" s="2">
+      <c r="G104" t="s" s="2">
         <v>711</v>
       </c>
-      <c r="G104" t="s" s="2">
-        <v>712</v>
-      </c>
       <c r="H104" t="s" s="2">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="I104" t="s" s="2">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>714</v>
+        <v>706</v>
       </c>
     </row>
     <row r="105">
@@ -6177,31 +6152,31 @@
         <v>19</v>
       </c>
       <c r="B105" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="C105" t="s" s="2">
+        <v>713</v>
+      </c>
+      <c r="D105" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="E105" t="s" s="2">
+        <v>713</v>
+      </c>
+      <c r="F105" t="s" s="2">
         <v>715</v>
       </c>
-      <c r="C105" t="s" s="2">
+      <c r="G105" t="s" s="2">
         <v>716</v>
       </c>
-      <c r="D105" t="s" s="2">
+      <c r="H105" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="I105" t="s" s="2">
         <v>717</v>
       </c>
-      <c r="E105" t="s" s="2">
-        <v>716</v>
-      </c>
-      <c r="F105" t="s" s="2">
-        <v>718</v>
-      </c>
-      <c r="G105" t="s" s="2">
-        <v>719</v>
-      </c>
-      <c r="H105" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="I105" t="s" s="2">
-        <v>713</v>
-      </c>
       <c r="J105" t="s" s="2">
-        <v>714</v>
+        <v>706</v>
       </c>
     </row>
     <row r="106">
@@ -6209,63 +6184,31 @@
         <v>19</v>
       </c>
       <c r="B106" t="s" s="2">
+        <v>718</v>
+      </c>
+      <c r="C106" t="s" s="2">
+        <v>719</v>
+      </c>
+      <c r="D106" t="s" s="2">
         <v>720</v>
       </c>
-      <c r="C106" t="s" s="2">
+      <c r="E106" t="s" s="2">
+        <v>719</v>
+      </c>
+      <c r="F106" t="s" s="2">
         <v>721</v>
       </c>
-      <c r="D106" t="s" s="2">
+      <c r="G106" t="s" s="2">
         <v>722</v>
       </c>
-      <c r="E106" t="s" s="2">
-        <v>721</v>
-      </c>
-      <c r="F106" t="s" s="2">
+      <c r="H106" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="I106" t="s" s="2">
         <v>723</v>
       </c>
-      <c r="G106" t="s" s="2">
-        <v>724</v>
-      </c>
-      <c r="H106" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="I106" t="s" s="2">
-        <v>725</v>
-      </c>
       <c r="J106" t="s" s="2">
-        <v>714</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="s" s="2">
-        <v>19</v>
-      </c>
-      <c r="B107" t="s" s="2">
-        <v>726</v>
-      </c>
-      <c r="C107" t="s" s="2">
-        <v>727</v>
-      </c>
-      <c r="D107" t="s" s="2">
-        <v>728</v>
-      </c>
-      <c r="E107" t="s" s="2">
-        <v>727</v>
-      </c>
-      <c r="F107" t="s" s="2">
-        <v>729</v>
-      </c>
-      <c r="G107" t="s" s="2">
-        <v>730</v>
-      </c>
-      <c r="H107" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="I107" t="s" s="2">
-        <v>731</v>
-      </c>
-      <c r="J107" t="s" s="2">
-        <v>714</v>
+        <v>706</v>
       </c>
     </row>
   </sheetData>
@@ -6277,18 +6220,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>732</v>
+        <v>724</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>734</v>
+        <v>726</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>735</v>
+        <v>727</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>19</v>
@@ -6302,10 +6245,10 @@
         <v>19</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>737</v>
+        <v>729</v>
       </c>
     </row>
     <row r="4">
@@ -6313,10 +6256,10 @@
         <v>19</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>737</v>
+        <v>729</v>
       </c>
     </row>
     <row r="5">
@@ -6324,10 +6267,10 @@
         <v>19</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>739</v>
+        <v>731</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>740</v>
+        <v>732</v>
       </c>
     </row>
     <row r="6">
@@ -6335,10 +6278,10 @@
         <v>19</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>741</v>
+        <v>733</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>742</v>
+        <v>734</v>
       </c>
     </row>
     <row r="7">
@@ -6346,10 +6289,10 @@
         <v>19</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>743</v>
+        <v>735</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>744</v>
+        <v>736</v>
       </c>
     </row>
     <row r="8">
@@ -6357,10 +6300,10 @@
         <v>19</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>745</v>
+        <v>737</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>746</v>
+        <v>738</v>
       </c>
     </row>
     <row r="9">
@@ -6368,10 +6311,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>747</v>
+        <v>739</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>748</v>
+        <v>740</v>
       </c>
     </row>
     <row r="10">
@@ -6379,10 +6322,10 @@
         <v>19</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>749</v>
+        <v>741</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>750</v>
+        <v>742</v>
       </c>
     </row>
     <row r="11">
@@ -6390,10 +6333,10 @@
         <v>19</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>751</v>
+        <v>743</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>752</v>
+        <v>744</v>
       </c>
     </row>
     <row r="12">
@@ -6401,10 +6344,10 @@
         <v>19</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>753</v>
+        <v>745</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>754</v>
+        <v>746</v>
       </c>
     </row>
     <row r="13">
@@ -6412,10 +6355,10 @@
         <v>19</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>755</v>
+        <v>747</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>756</v>
+        <v>748</v>
       </c>
     </row>
     <row r="14">
@@ -6423,10 +6366,10 @@
         <v>19</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>757</v>
+        <v>749</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>758</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15">
@@ -6434,10 +6377,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>759</v>
+        <v>751</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>760</v>
+        <v>752</v>
       </c>
     </row>
     <row r="16">
@@ -6445,10 +6388,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>761</v>
+        <v>753</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>762</v>
+        <v>754</v>
       </c>
     </row>
     <row r="17">
@@ -6456,10 +6399,10 @@
         <v>19</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>763</v>
+        <v>755</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>764</v>
+        <v>756</v>
       </c>
     </row>
     <row r="18">
@@ -6467,10 +6410,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>765</v>
+        <v>757</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>766</v>
+        <v>758</v>
       </c>
     </row>
     <row r="19">
@@ -6478,10 +6421,10 @@
         <v>19</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>767</v>
+        <v>759</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>768</v>
+        <v>760</v>
       </c>
     </row>
     <row r="20">
@@ -6489,10 +6432,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>769</v>
+        <v>761</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>770</v>
+        <v>762</v>
       </c>
     </row>
     <row r="21">
@@ -6500,10 +6443,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>771</v>
+        <v>763</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>772</v>
+        <v>764</v>
       </c>
     </row>
     <row r="22">
@@ -6511,10 +6454,10 @@
         <v>19</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>773</v>
+        <v>765</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>774</v>
+        <v>766</v>
       </c>
     </row>
     <row r="23">
@@ -6522,10 +6465,10 @@
         <v>19</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>775</v>
+        <v>767</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>776</v>
+        <v>768</v>
       </c>
     </row>
     <row r="24">
@@ -6533,10 +6476,10 @@
         <v>19</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>777</v>
+        <v>769</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>778</v>
+        <v>770</v>
       </c>
     </row>
     <row r="25">
@@ -6544,10 +6487,10 @@
         <v>19</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>779</v>
+        <v>771</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>780</v>
+        <v>772</v>
       </c>
     </row>
     <row r="26">
@@ -6555,10 +6498,10 @@
         <v>19</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>781</v>
+        <v>773</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>782</v>
+        <v>774</v>
       </c>
     </row>
     <row r="27">
@@ -6566,10 +6509,10 @@
         <v>19</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>783</v>
+        <v>775</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>784</v>
+        <v>776</v>
       </c>
     </row>
     <row r="28">
@@ -6577,10 +6520,10 @@
         <v>19</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>785</v>
+        <v>777</v>
       </c>
       <c r="C28" t="s" s="2">
-        <v>786</v>
+        <v>778</v>
       </c>
     </row>
     <row r="29">
@@ -6588,10 +6531,10 @@
         <v>19</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>787</v>
+        <v>779</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>788</v>
+        <v>780</v>
       </c>
     </row>
     <row r="30">
@@ -6599,10 +6542,10 @@
         <v>19</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>789</v>
+        <v>781</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>790</v>
+        <v>782</v>
       </c>
     </row>
     <row r="31">
@@ -6610,10 +6553,10 @@
         <v>19</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>791</v>
+        <v>783</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>792</v>
+        <v>784</v>
       </c>
     </row>
     <row r="32">
@@ -6621,10 +6564,10 @@
         <v>19</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>793</v>
+        <v>785</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>794</v>
+        <v>786</v>
       </c>
     </row>
     <row r="33">
@@ -6632,10 +6575,10 @@
         <v>19</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>795</v>
+        <v>787</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>796</v>
+        <v>788</v>
       </c>
     </row>
     <row r="34">
@@ -6643,10 +6586,10 @@
         <v>19</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>798</v>
+        <v>790</v>
       </c>
     </row>
     <row r="35">
@@ -6654,10 +6597,10 @@
         <v>19</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>800</v>
+        <v>792</v>
       </c>
     </row>
     <row r="36">
@@ -6665,10 +6608,10 @@
         <v>19</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>801</v>
+        <v>793</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>802</v>
+        <v>794</v>
       </c>
     </row>
     <row r="37">
@@ -6676,10 +6619,10 @@
         <v>19</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>803</v>
+        <v>795</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>804</v>
+        <v>796</v>
       </c>
     </row>
     <row r="38">
@@ -6687,10 +6630,10 @@
         <v>19</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>805</v>
+        <v>797</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>806</v>
+        <v>798</v>
       </c>
     </row>
     <row r="39">
@@ -6698,10 +6641,10 @@
         <v>19</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>807</v>
+        <v>799</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>808</v>
+        <v>800</v>
       </c>
     </row>
     <row r="40">
@@ -6709,10 +6652,10 @@
         <v>19</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>809</v>
+        <v>801</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>810</v>
+        <v>802</v>
       </c>
     </row>
     <row r="41">
@@ -6720,10 +6663,10 @@
         <v>19</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>811</v>
+        <v>803</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>812</v>
+        <v>804</v>
       </c>
     </row>
     <row r="42">
@@ -6731,10 +6674,10 @@
         <v>19</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>813</v>
+        <v>805</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>814</v>
+        <v>806</v>
       </c>
     </row>
     <row r="43">
@@ -6742,10 +6685,10 @@
         <v>19</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>815</v>
+        <v>807</v>
       </c>
       <c r="C43" t="s" s="2">
-        <v>816</v>
+        <v>808</v>
       </c>
     </row>
     <row r="44">
@@ -6753,10 +6696,10 @@
         <v>19</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>817</v>
+        <v>809</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>818</v>
+        <v>810</v>
       </c>
     </row>
     <row r="45">
@@ -6764,10 +6707,10 @@
         <v>19</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>819</v>
+        <v>811</v>
       </c>
       <c r="C45" t="s" s="2">
-        <v>820</v>
+        <v>812</v>
       </c>
     </row>
     <row r="46">
@@ -6775,10 +6718,10 @@
         <v>19</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>821</v>
+        <v>813</v>
       </c>
       <c r="C46" t="s" s="2">
-        <v>822</v>
+        <v>814</v>
       </c>
     </row>
     <row r="47">
@@ -6786,10 +6729,10 @@
         <v>19</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>823</v>
+        <v>815</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>824</v>
+        <v>816</v>
       </c>
     </row>
     <row r="48">
@@ -6797,10 +6740,10 @@
         <v>19</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>825</v>
+        <v>817</v>
       </c>
       <c r="C48" t="s" s="2">
-        <v>826</v>
+        <v>818</v>
       </c>
     </row>
     <row r="49">
@@ -6808,10 +6751,10 @@
         <v>19</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>827</v>
+        <v>819</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>828</v>
+        <v>820</v>
       </c>
     </row>
     <row r="50">
@@ -6819,10 +6762,10 @@
         <v>19</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>829</v>
+        <v>821</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>830</v>
+        <v>822</v>
       </c>
     </row>
     <row r="51">
@@ -6830,10 +6773,10 @@
         <v>19</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>831</v>
+        <v>823</v>
       </c>
       <c r="C51" t="s" s="2">
-        <v>832</v>
+        <v>824</v>
       </c>
     </row>
     <row r="52">
@@ -6844,7 +6787,7 @@
         <v>233</v>
       </c>
       <c r="C52" t="s" s="2">
-        <v>833</v>
+        <v>825</v>
       </c>
     </row>
     <row r="53">
@@ -6855,7 +6798,7 @@
         <v>462</v>
       </c>
       <c r="C53" t="s" s="2">
-        <v>834</v>
+        <v>826</v>
       </c>
     </row>
     <row r="54">
@@ -6863,10 +6806,10 @@
         <v>19</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>835</v>
+        <v>827</v>
       </c>
       <c r="C54" t="s" s="2">
-        <v>836</v>
+        <v>828</v>
       </c>
     </row>
     <row r="55">
@@ -6874,10 +6817,10 @@
         <v>19</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>837</v>
+        <v>829</v>
       </c>
       <c r="C55" t="s" s="2">
-        <v>838</v>
+        <v>830</v>
       </c>
     </row>
     <row r="56">
@@ -6885,10 +6828,10 @@
         <v>19</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>839</v>
+        <v>831</v>
       </c>
       <c r="C56" t="s" s="2">
-        <v>840</v>
+        <v>832</v>
       </c>
     </row>
     <row r="57">
@@ -6896,10 +6839,10 @@
         <v>19</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>841</v>
+        <v>833</v>
       </c>
       <c r="C57" t="s" s="2">
-        <v>842</v>
+        <v>834</v>
       </c>
     </row>
     <row r="58">
@@ -6907,10 +6850,10 @@
         <v>19</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>843</v>
+        <v>835</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>844</v>
+        <v>836</v>
       </c>
     </row>
     <row r="59">
@@ -6918,10 +6861,10 @@
         <v>19</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>845</v>
+        <v>837</v>
       </c>
       <c r="C59" t="s" s="2">
-        <v>846</v>
+        <v>838</v>
       </c>
     </row>
     <row r="60">
@@ -6929,10 +6872,10 @@
         <v>19</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>847</v>
+        <v>839</v>
       </c>
       <c r="C60" t="s" s="2">
-        <v>848</v>
+        <v>840</v>
       </c>
     </row>
     <row r="61">
@@ -6940,10 +6883,10 @@
         <v>19</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>849</v>
+        <v>841</v>
       </c>
       <c r="C61" t="s" s="2">
-        <v>850</v>
+        <v>842</v>
       </c>
     </row>
     <row r="62">
@@ -6951,10 +6894,10 @@
         <v>19</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>851</v>
+        <v>843</v>
       </c>
       <c r="C62" t="s" s="2">
-        <v>852</v>
+        <v>844</v>
       </c>
     </row>
     <row r="63">
@@ -6962,10 +6905,10 @@
         <v>19</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>853</v>
+        <v>845</v>
       </c>
       <c r="C63" t="s" s="2">
-        <v>854</v>
+        <v>846</v>
       </c>
     </row>
     <row r="64">
@@ -6976,7 +6919,7 @@
         <v>550</v>
       </c>
       <c r="C64" t="s" s="2">
-        <v>855</v>
+        <v>847</v>
       </c>
     </row>
     <row r="65">
@@ -6992,7 +6935,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>856</v>
+        <v>848</v>
       </c>
       <c r="B66" t="s" s="2">
         <v>19</v>
@@ -7006,10 +6949,10 @@
         <v>19</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="C67" t="s" s="2">
-        <v>858</v>
+        <v>850</v>
       </c>
     </row>
     <row r="68">
@@ -7017,10 +6960,10 @@
         <v>19</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>859</v>
+        <v>851</v>
       </c>
       <c r="C68" t="s" s="2">
-        <v>860</v>
+        <v>852</v>
       </c>
     </row>
     <row r="69">
@@ -7028,10 +6971,10 @@
         <v>19</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>861</v>
+        <v>853</v>
       </c>
       <c r="C69" t="s" s="2">
-        <v>862</v>
+        <v>854</v>
       </c>
     </row>
     <row r="70">
@@ -7039,10 +6982,10 @@
         <v>19</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>863</v>
+        <v>855</v>
       </c>
       <c r="C70" t="s" s="2">
-        <v>864</v>
+        <v>856</v>
       </c>
     </row>
     <row r="71">
@@ -7050,10 +6993,10 @@
         <v>19</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>865</v>
+        <v>857</v>
       </c>
       <c r="C71" t="s" s="2">
-        <v>866</v>
+        <v>858</v>
       </c>
     </row>
     <row r="72">
@@ -7061,10 +7004,10 @@
         <v>19</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>867</v>
+        <v>859</v>
       </c>
       <c r="C72" t="s" s="2">
-        <v>868</v>
+        <v>860</v>
       </c>
     </row>
     <row r="73">
@@ -7072,10 +7015,10 @@
         <v>19</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>869</v>
+        <v>861</v>
       </c>
       <c r="C73" t="s" s="2">
-        <v>870</v>
+        <v>862</v>
       </c>
     </row>
     <row r="74">
@@ -7083,10 +7026,10 @@
         <v>19</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>871</v>
+        <v>863</v>
       </c>
       <c r="C74" t="s" s="2">
-        <v>872</v>
+        <v>864</v>
       </c>
     </row>
     <row r="75">
@@ -7094,10 +7037,10 @@
         <v>19</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>873</v>
+        <v>865</v>
       </c>
       <c r="C75" t="s" s="2">
-        <v>874</v>
+        <v>866</v>
       </c>
     </row>
     <row r="76">
@@ -7105,10 +7048,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>875</v>
+        <v>867</v>
       </c>
       <c r="C76" t="s" s="2">
-        <v>876</v>
+        <v>868</v>
       </c>
     </row>
     <row r="77">
@@ -7116,10 +7059,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>877</v>
+        <v>869</v>
       </c>
       <c r="C77" t="s" s="2">
-        <v>878</v>
+        <v>870</v>
       </c>
     </row>
     <row r="78">
@@ -7127,10 +7070,10 @@
         <v>19</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>879</v>
+        <v>871</v>
       </c>
       <c r="C78" t="s" s="2">
-        <v>880</v>
+        <v>872</v>
       </c>
     </row>
     <row r="79">
@@ -7138,10 +7081,10 @@
         <v>19</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>881</v>
+        <v>873</v>
       </c>
       <c r="C79" t="s" s="2">
-        <v>882</v>
+        <v>874</v>
       </c>
     </row>
     <row r="80">
@@ -7149,10 +7092,10 @@
         <v>19</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="C80" t="s" s="2">
-        <v>884</v>
+        <v>876</v>
       </c>
     </row>
   </sheetData>
@@ -7167,43 +7110,43 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>885</v>
+        <v>877</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>886</v>
+        <v>878</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>887</v>
+        <v>879</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>693</v>
+        <v>685</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>888</v>
+        <v>880</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>700</v>
+        <v>692</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>889</v>
+        <v>881</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>705</v>
+        <v>697</v>
       </c>
     </row>
   </sheetData>
@@ -7227,58 +7170,58 @@
         <v>4</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>890</v>
+        <v>882</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>691</v>
+        <v>683</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>695</v>
+        <v>687</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>698</v>
+        <v>690</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>695</v>
+        <v>687</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>706</v>
+        <v>698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>